<commit_message>
docs: the daily log Sep 17 Excel study
</commit_message>
<xml_diff>
--- a/tea_shop_model.xlsx
+++ b/tea_shop_model.xlsx
@@ -9,11 +9,12 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="9192" windowHeight="2988"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="9192" windowHeight="2988" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="方案摘要" sheetId="2" r:id="rId1"/>
     <sheet name="Model1" sheetId="1" r:id="rId2"/>
+    <sheet name="Demand_Curve" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="75">
   <si>
     <t>初始月租金</t>
     <phoneticPr fontId="2" type="noConversion"/>
@@ -262,6 +263,18 @@
   </si>
   <si>
     <t>每组方案的可变单元格均以灰色底纹突出显示。</t>
+  </si>
+  <si>
+    <t>Price</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Quantity</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>PED</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -505,6 +518,1138 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="zh-CN"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:layout/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="zh-CN"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Demand Curve for milk tea</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Demand_Curve!$B$2:$B$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>150</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>200</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>250</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>300</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>350</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>400</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>450</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>500</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>550</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Demand_Curve!$A$2:$A$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>6</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-A2B5-4BAC-97D0-44981B88D339}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="415067312"/>
+        <c:axId val="415067968"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="415067312"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:layout/>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="zh-CN"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="zh-CN"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="415067968"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="415067968"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="zh-CN"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="415067312"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="zh-CN"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+  <c:userShapes r:id="rId3"/>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>53340</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>87630</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>358140</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>26670</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="图表 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>403860</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>68580</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1102097" cy="412951"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="文本框 2"/>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8938260" y="3223260"/>
+          <a:ext cx="1102097" cy="412951"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="t">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1100"/>
+            <a:t>Inelastic(PED&lt;1</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="zh-CN" altLang="en-US" sz="1100"/>
+            <a:t>）</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:userShapes xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
+    <cdr:from>
+      <cdr:x>0.22333</cdr:x>
+      <cdr:y>0.11528</cdr:y>
+    </cdr:from>
+    <cdr:to>
+      <cdr:x>0.39333</cdr:x>
+      <cdr:y>0.19861</cdr:y>
+    </cdr:to>
+    <cdr:sp macro="" textlink="">
+      <cdr:nvSpPr>
+        <cdr:cNvPr id="4" name="文本框 3"/>
+        <cdr:cNvSpPr txBox="1"/>
+      </cdr:nvSpPr>
+      <cdr:spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="1021080" y="316230"/>
+          <a:ext cx="777240" cy="228600"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </cdr:spPr>
+      <cdr:txBody>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" vertOverflow="clip" wrap="none" rtlCol="0"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:endParaRPr lang="zh-CN" altLang="en-US" sz="1100"/>
+        </a:p>
+      </cdr:txBody>
+    </cdr:sp>
+  </cdr:relSizeAnchor>
+  <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
+    <cdr:from>
+      <cdr:x>0.23</cdr:x>
+      <cdr:y>0.12639</cdr:y>
+    </cdr:from>
+    <cdr:to>
+      <cdr:x>0.37333</cdr:x>
+      <cdr:y>0.19583</cdr:y>
+    </cdr:to>
+    <cdr:sp macro="" textlink="">
+      <cdr:nvSpPr>
+        <cdr:cNvPr id="5" name="文本框 4"/>
+        <cdr:cNvSpPr txBox="1"/>
+      </cdr:nvSpPr>
+      <cdr:spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="1051560" y="346710"/>
+          <a:ext cx="655320" cy="190500"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </cdr:spPr>
+      <cdr:txBody>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" vertOverflow="clip" wrap="none" rtlCol="0"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:endParaRPr lang="zh-CN" altLang="en-US" sz="1100"/>
+        </a:p>
+      </cdr:txBody>
+    </cdr:sp>
+  </cdr:relSizeAnchor>
+  <cdr:relSizeAnchor xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing">
+    <cdr:from>
+      <cdr:x>0.21167</cdr:x>
+      <cdr:y>0.15139</cdr:y>
+    </cdr:from>
+    <cdr:to>
+      <cdr:x>0.42667</cdr:x>
+      <cdr:y>0.24306</cdr:y>
+    </cdr:to>
+    <cdr:sp macro="" textlink="">
+      <cdr:nvSpPr>
+        <cdr:cNvPr id="6" name="文本框 5"/>
+        <cdr:cNvSpPr txBox="1"/>
+      </cdr:nvSpPr>
+      <cdr:spPr>
+        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:off x="967740" y="415290"/>
+          <a:ext cx="982980" cy="251460"/>
+        </a:xfrm>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </cdr:spPr>
+      <cdr:txBody>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" vertOverflow="clip" wrap="none" rtlCol="0"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:r>
+            <a:rPr lang="en-US" altLang="zh-CN" sz="1100"/>
+            <a:t>Elasitc (PED&gt;1)</a:t>
+          </a:r>
+        </a:p>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:endParaRPr lang="zh-CN" altLang="en-US" sz="1100"/>
+        </a:p>
+      </cdr:txBody>
+    </cdr:sp>
+  </cdr:relSizeAnchor>
+</c:userShapes>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -990,7 +2135,7 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>15</v>
+        <v>30.383651873447796</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
@@ -998,7 +2143,7 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>200</v>
+        <v>80</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
@@ -1015,7 +2160,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="1">
-        <v>0.05</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
@@ -1023,7 +2168,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="1">
-        <v>0</v>
+        <v>-0.15</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
@@ -1075,27 +2220,27 @@
       </c>
       <c r="D11">
         <f>$B$5*30</f>
-        <v>6000</v>
+        <v>2400</v>
       </c>
       <c r="E11">
         <f>$B$4*D11</f>
-        <v>90000</v>
+        <v>72920.764496274714</v>
       </c>
       <c r="F11">
         <f>$B$3*D11</f>
-        <v>18000</v>
+        <v>7200</v>
       </c>
       <c r="G11">
         <f>B11+C11+F11</f>
-        <v>53000</v>
+        <v>42200</v>
       </c>
       <c r="H11">
         <f>E11-G11</f>
-        <v>37000</v>
+        <v>30720.764496274714</v>
       </c>
       <c r="I11">
         <f>H11</f>
-        <v>37000</v>
+        <v>30720.764496274714</v>
       </c>
       <c r="J11" t="str">
         <f>IF(H11&gt;50000,"优秀",IF(H11&gt;0,"盈利",IF(H11=0,"保本","亏损")))</f>
@@ -1103,7 +2248,7 @@
       </c>
       <c r="K11">
         <f>IF(H11&lt;0,0,IF(D11&gt;4500,H11*0.05,IF(D11&gt;3500,H11*0.02,0)))</f>
-        <v>1850</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
@@ -1120,27 +2265,27 @@
       </c>
       <c r="D12">
         <f t="shared" ref="D12:D22" si="2">$B$5*30</f>
-        <v>6000</v>
+        <v>2400</v>
       </c>
       <c r="E12">
         <f t="shared" ref="E12:E22" si="3">$B$4*D12</f>
-        <v>90000</v>
+        <v>72920.764496274714</v>
       </c>
       <c r="F12">
         <f t="shared" ref="F12:F22" si="4">$B$3*D12</f>
-        <v>18000</v>
+        <v>7200</v>
       </c>
       <c r="G12">
         <f t="shared" ref="G12:G22" si="5">B12+C12+F12</f>
-        <v>53000</v>
+        <v>42200</v>
       </c>
       <c r="H12">
         <f t="shared" ref="H12:H22" si="6">E12-G12</f>
-        <v>37000</v>
+        <v>30720.764496274714</v>
       </c>
       <c r="I12">
         <f>H12+I11</f>
-        <v>74000</v>
+        <v>61441.528992549429</v>
       </c>
       <c r="J12" t="str">
         <f t="shared" ref="J12:J46" si="7">IF(H12&gt;50000,"优秀",IF(H12&gt;0,"盈利",IF(H12=0,"保本","亏损")))</f>
@@ -1148,7 +2293,7 @@
       </c>
       <c r="K12">
         <f t="shared" ref="K12:K46" si="8">IF(H12&lt;0,0,IF(D12&gt;4500,H12*0.05,IF(D12&gt;3500,H12*0.02,0)))</f>
-        <v>1850</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
@@ -1165,27 +2310,27 @@
       </c>
       <c r="D13">
         <f t="shared" si="2"/>
-        <v>6000</v>
+        <v>2400</v>
       </c>
       <c r="E13">
         <f t="shared" si="3"/>
-        <v>90000</v>
+        <v>72920.764496274714</v>
       </c>
       <c r="F13">
         <f t="shared" si="4"/>
-        <v>18000</v>
+        <v>7200</v>
       </c>
       <c r="G13">
         <f t="shared" si="5"/>
-        <v>53000</v>
+        <v>42200</v>
       </c>
       <c r="H13">
         <f t="shared" si="6"/>
-        <v>37000</v>
+        <v>30720.764496274714</v>
       </c>
       <c r="I13">
         <f t="shared" ref="I13:I46" si="9">H13+I12</f>
-        <v>111000</v>
+        <v>92162.293488824143</v>
       </c>
       <c r="J13" t="str">
         <f t="shared" si="7"/>
@@ -1193,7 +2338,7 @@
       </c>
       <c r="K13">
         <f t="shared" si="8"/>
-        <v>1850</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
@@ -1210,27 +2355,27 @@
       </c>
       <c r="D14">
         <f t="shared" si="2"/>
-        <v>6000</v>
+        <v>2400</v>
       </c>
       <c r="E14">
         <f t="shared" si="3"/>
-        <v>90000</v>
+        <v>72920.764496274714</v>
       </c>
       <c r="F14">
         <f t="shared" si="4"/>
-        <v>18000</v>
+        <v>7200</v>
       </c>
       <c r="G14">
         <f t="shared" si="5"/>
-        <v>53000</v>
+        <v>42200</v>
       </c>
       <c r="H14">
         <f t="shared" si="6"/>
-        <v>37000</v>
+        <v>30720.764496274714</v>
       </c>
       <c r="I14">
         <f t="shared" si="9"/>
-        <v>148000</v>
+        <v>122883.05798509886</v>
       </c>
       <c r="J14" t="str">
         <f t="shared" si="7"/>
@@ -1238,7 +2383,7 @@
       </c>
       <c r="K14">
         <f t="shared" si="8"/>
-        <v>1850</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
@@ -1255,27 +2400,27 @@
       </c>
       <c r="D15">
         <f t="shared" si="2"/>
-        <v>6000</v>
+        <v>2400</v>
       </c>
       <c r="E15">
         <f t="shared" si="3"/>
-        <v>90000</v>
+        <v>72920.764496274714</v>
       </c>
       <c r="F15">
         <f t="shared" si="4"/>
-        <v>18000</v>
+        <v>7200</v>
       </c>
       <c r="G15">
         <f t="shared" si="5"/>
-        <v>53000</v>
+        <v>42200</v>
       </c>
       <c r="H15">
         <f t="shared" si="6"/>
-        <v>37000</v>
+        <v>30720.764496274714</v>
       </c>
       <c r="I15">
         <f t="shared" si="9"/>
-        <v>185000</v>
+        <v>153603.82248137356</v>
       </c>
       <c r="J15" t="str">
         <f t="shared" si="7"/>
@@ -1283,7 +2428,7 @@
       </c>
       <c r="K15">
         <f t="shared" si="8"/>
-        <v>1850</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
@@ -1300,27 +2445,27 @@
       </c>
       <c r="D16">
         <f t="shared" si="2"/>
-        <v>6000</v>
+        <v>2400</v>
       </c>
       <c r="E16">
         <f t="shared" si="3"/>
-        <v>90000</v>
+        <v>72920.764496274714</v>
       </c>
       <c r="F16">
         <f t="shared" si="4"/>
-        <v>18000</v>
+        <v>7200</v>
       </c>
       <c r="G16">
         <f t="shared" si="5"/>
-        <v>53000</v>
+        <v>42200</v>
       </c>
       <c r="H16">
         <f t="shared" si="6"/>
-        <v>37000</v>
+        <v>30720.764496274714</v>
       </c>
       <c r="I16">
         <f t="shared" si="9"/>
-        <v>222000</v>
+        <v>184324.58697764826</v>
       </c>
       <c r="J16" t="str">
         <f t="shared" si="7"/>
@@ -1328,7 +2473,7 @@
       </c>
       <c r="K16">
         <f t="shared" si="8"/>
-        <v>1850</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
@@ -1345,27 +2490,27 @@
       </c>
       <c r="D17">
         <f t="shared" si="2"/>
-        <v>6000</v>
+        <v>2400</v>
       </c>
       <c r="E17">
         <f t="shared" si="3"/>
-        <v>90000</v>
+        <v>72920.764496274714</v>
       </c>
       <c r="F17">
         <f t="shared" si="4"/>
-        <v>18000</v>
+        <v>7200</v>
       </c>
       <c r="G17">
         <f t="shared" si="5"/>
-        <v>53000</v>
+        <v>42200</v>
       </c>
       <c r="H17">
         <f t="shared" si="6"/>
-        <v>37000</v>
+        <v>30720.764496274714</v>
       </c>
       <c r="I17">
         <f t="shared" si="9"/>
-        <v>259000</v>
+        <v>215045.35147392296</v>
       </c>
       <c r="J17" t="str">
         <f t="shared" si="7"/>
@@ -1373,7 +2518,7 @@
       </c>
       <c r="K17">
         <f t="shared" si="8"/>
-        <v>1850</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
@@ -1390,27 +2535,27 @@
       </c>
       <c r="D18">
         <f t="shared" si="2"/>
-        <v>6000</v>
+        <v>2400</v>
       </c>
       <c r="E18">
         <f t="shared" si="3"/>
-        <v>90000</v>
+        <v>72920.764496274714</v>
       </c>
       <c r="F18">
         <f t="shared" si="4"/>
-        <v>18000</v>
+        <v>7200</v>
       </c>
       <c r="G18">
         <f t="shared" si="5"/>
-        <v>53000</v>
+        <v>42200</v>
       </c>
       <c r="H18">
         <f t="shared" si="6"/>
-        <v>37000</v>
+        <v>30720.764496274714</v>
       </c>
       <c r="I18">
         <f t="shared" si="9"/>
-        <v>296000</v>
+        <v>245766.11597019766</v>
       </c>
       <c r="J18" t="str">
         <f t="shared" si="7"/>
@@ -1418,7 +2563,7 @@
       </c>
       <c r="K18">
         <f t="shared" si="8"/>
-        <v>1850</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
@@ -1435,27 +2580,27 @@
       </c>
       <c r="D19">
         <f t="shared" si="2"/>
-        <v>6000</v>
+        <v>2400</v>
       </c>
       <c r="E19">
         <f t="shared" si="3"/>
-        <v>90000</v>
+        <v>72920.764496274714</v>
       </c>
       <c r="F19">
         <f t="shared" si="4"/>
-        <v>18000</v>
+        <v>7200</v>
       </c>
       <c r="G19">
         <f t="shared" si="5"/>
-        <v>53000</v>
+        <v>42200</v>
       </c>
       <c r="H19">
         <f t="shared" si="6"/>
-        <v>37000</v>
+        <v>30720.764496274714</v>
       </c>
       <c r="I19">
         <f t="shared" si="9"/>
-        <v>333000</v>
+        <v>276486.88046647236</v>
       </c>
       <c r="J19" t="str">
         <f t="shared" si="7"/>
@@ -1463,7 +2608,7 @@
       </c>
       <c r="K19">
         <f t="shared" si="8"/>
-        <v>1850</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
@@ -1480,27 +2625,27 @@
       </c>
       <c r="D20">
         <f t="shared" si="2"/>
-        <v>6000</v>
+        <v>2400</v>
       </c>
       <c r="E20">
         <f t="shared" si="3"/>
-        <v>90000</v>
+        <v>72920.764496274714</v>
       </c>
       <c r="F20">
         <f t="shared" si="4"/>
-        <v>18000</v>
+        <v>7200</v>
       </c>
       <c r="G20">
         <f t="shared" si="5"/>
-        <v>53000</v>
+        <v>42200</v>
       </c>
       <c r="H20">
         <f t="shared" si="6"/>
-        <v>37000</v>
+        <v>30720.764496274714</v>
       </c>
       <c r="I20">
         <f t="shared" si="9"/>
-        <v>370000</v>
+        <v>307207.64496274706</v>
       </c>
       <c r="J20" t="str">
         <f t="shared" si="7"/>
@@ -1508,7 +2653,7 @@
       </c>
       <c r="K20">
         <f t="shared" si="8"/>
-        <v>1850</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
@@ -1525,27 +2670,27 @@
       </c>
       <c r="D21">
         <f t="shared" si="2"/>
-        <v>6000</v>
+        <v>2400</v>
       </c>
       <c r="E21">
         <f t="shared" si="3"/>
-        <v>90000</v>
+        <v>72920.764496274714</v>
       </c>
       <c r="F21">
         <f t="shared" si="4"/>
-        <v>18000</v>
+        <v>7200</v>
       </c>
       <c r="G21">
         <f t="shared" si="5"/>
-        <v>53000</v>
+        <v>42200</v>
       </c>
       <c r="H21">
         <f t="shared" si="6"/>
-        <v>37000</v>
+        <v>30720.764496274714</v>
       </c>
       <c r="I21">
         <f t="shared" si="9"/>
-        <v>407000</v>
+        <v>337928.40945902176</v>
       </c>
       <c r="J21" t="str">
         <f t="shared" si="7"/>
@@ -1553,7 +2698,7 @@
       </c>
       <c r="K21">
         <f t="shared" si="8"/>
-        <v>1850</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
@@ -1570,27 +2715,27 @@
       </c>
       <c r="D22">
         <f t="shared" si="2"/>
-        <v>6000</v>
+        <v>2400</v>
       </c>
       <c r="E22">
         <f t="shared" si="3"/>
-        <v>90000</v>
+        <v>72920.764496274714</v>
       </c>
       <c r="F22">
         <f t="shared" si="4"/>
-        <v>18000</v>
+        <v>7200</v>
       </c>
       <c r="G22">
         <f t="shared" si="5"/>
-        <v>53000</v>
+        <v>42200</v>
       </c>
       <c r="H22">
         <f t="shared" si="6"/>
-        <v>37000</v>
+        <v>30720.764496274714</v>
       </c>
       <c r="I22">
         <f t="shared" si="9"/>
-        <v>444000</v>
+        <v>368649.17395529646</v>
       </c>
       <c r="J22" t="str">
         <f t="shared" si="7"/>
@@ -1598,7 +2743,7 @@
       </c>
       <c r="K22">
         <f t="shared" si="8"/>
-        <v>1850</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
@@ -1607,35 +2752,35 @@
       </c>
       <c r="B23">
         <f>$B$1*(1+$B$7)</f>
-        <v>15750</v>
+        <v>18000</v>
       </c>
       <c r="C23">
         <f>$B$2*(1+$B$7)</f>
-        <v>21000</v>
+        <v>24000</v>
       </c>
       <c r="D23">
         <f>$B$5*30*(1+$B$8)</f>
-        <v>6000</v>
+        <v>2040</v>
       </c>
       <c r="E23">
         <f>$B$4*D23</f>
-        <v>90000</v>
+        <v>61982.649821833504</v>
       </c>
       <c r="F23">
         <f>$B$3*D23</f>
-        <v>18000</v>
+        <v>6120</v>
       </c>
       <c r="G23">
         <f>B23+C23+F23</f>
-        <v>54750</v>
+        <v>48120</v>
       </c>
       <c r="H23">
         <f>E23-G23</f>
-        <v>35250</v>
+        <v>13862.649821833504</v>
       </c>
       <c r="I23">
         <f t="shared" si="9"/>
-        <v>479250</v>
+        <v>382511.82377712999</v>
       </c>
       <c r="J23" t="str">
         <f t="shared" si="7"/>
@@ -1643,7 +2788,7 @@
       </c>
       <c r="K23">
         <f t="shared" si="8"/>
-        <v>1762.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
@@ -1652,35 +2797,35 @@
       </c>
       <c r="B24">
         <f t="shared" ref="B24:B34" si="10">$B$1*(1+$B$7)</f>
-        <v>15750</v>
+        <v>18000</v>
       </c>
       <c r="C24">
         <f t="shared" ref="C24:C34" si="11">$B$2*(1+$B$7)</f>
-        <v>21000</v>
+        <v>24000</v>
       </c>
       <c r="D24">
         <f t="shared" ref="D24:D34" si="12">$B$5*30*(1+$B$8)</f>
-        <v>6000</v>
+        <v>2040</v>
       </c>
       <c r="E24">
         <f t="shared" ref="E24:E46" si="13">$B$4*D24</f>
-        <v>90000</v>
+        <v>61982.649821833504</v>
       </c>
       <c r="F24">
         <f t="shared" ref="F24:F46" si="14">$B$3*D24</f>
-        <v>18000</v>
+        <v>6120</v>
       </c>
       <c r="G24">
         <f t="shared" ref="G24:G46" si="15">B24+C24+F24</f>
-        <v>54750</v>
+        <v>48120</v>
       </c>
       <c r="H24">
         <f t="shared" ref="H24:H46" si="16">E24-G24</f>
-        <v>35250</v>
+        <v>13862.649821833504</v>
       </c>
       <c r="I24">
         <f t="shared" si="9"/>
-        <v>514500</v>
+        <v>396374.47359896346</v>
       </c>
       <c r="J24" t="str">
         <f t="shared" si="7"/>
@@ -1688,7 +2833,7 @@
       </c>
       <c r="K24">
         <f t="shared" si="8"/>
-        <v>1762.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
@@ -1697,35 +2842,35 @@
       </c>
       <c r="B25">
         <f t="shared" si="10"/>
-        <v>15750</v>
+        <v>18000</v>
       </c>
       <c r="C25">
         <f t="shared" si="11"/>
-        <v>21000</v>
+        <v>24000</v>
       </c>
       <c r="D25">
         <f t="shared" si="12"/>
-        <v>6000</v>
+        <v>2040</v>
       </c>
       <c r="E25">
         <f t="shared" si="13"/>
-        <v>90000</v>
+        <v>61982.649821833504</v>
       </c>
       <c r="F25">
         <f t="shared" si="14"/>
-        <v>18000</v>
+        <v>6120</v>
       </c>
       <c r="G25">
         <f t="shared" si="15"/>
-        <v>54750</v>
+        <v>48120</v>
       </c>
       <c r="H25">
         <f t="shared" si="16"/>
-        <v>35250</v>
+        <v>13862.649821833504</v>
       </c>
       <c r="I25">
         <f t="shared" si="9"/>
-        <v>549750</v>
+        <v>410237.12342079694</v>
       </c>
       <c r="J25" t="str">
         <f t="shared" si="7"/>
@@ -1733,7 +2878,7 @@
       </c>
       <c r="K25">
         <f t="shared" si="8"/>
-        <v>1762.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
@@ -1742,35 +2887,35 @@
       </c>
       <c r="B26">
         <f t="shared" si="10"/>
-        <v>15750</v>
+        <v>18000</v>
       </c>
       <c r="C26">
         <f t="shared" si="11"/>
-        <v>21000</v>
+        <v>24000</v>
       </c>
       <c r="D26">
         <f t="shared" si="12"/>
-        <v>6000</v>
+        <v>2040</v>
       </c>
       <c r="E26">
         <f t="shared" si="13"/>
-        <v>90000</v>
+        <v>61982.649821833504</v>
       </c>
       <c r="F26">
         <f t="shared" si="14"/>
-        <v>18000</v>
+        <v>6120</v>
       </c>
       <c r="G26">
         <f t="shared" si="15"/>
-        <v>54750</v>
+        <v>48120</v>
       </c>
       <c r="H26">
         <f t="shared" si="16"/>
-        <v>35250</v>
+        <v>13862.649821833504</v>
       </c>
       <c r="I26">
         <f t="shared" si="9"/>
-        <v>585000</v>
+        <v>424099.77324263041</v>
       </c>
       <c r="J26" t="str">
         <f t="shared" si="7"/>
@@ -1778,7 +2923,7 @@
       </c>
       <c r="K26">
         <f t="shared" si="8"/>
-        <v>1762.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
@@ -1787,35 +2932,35 @@
       </c>
       <c r="B27">
         <f t="shared" si="10"/>
-        <v>15750</v>
+        <v>18000</v>
       </c>
       <c r="C27">
         <f t="shared" si="11"/>
-        <v>21000</v>
+        <v>24000</v>
       </c>
       <c r="D27">
         <f t="shared" si="12"/>
-        <v>6000</v>
+        <v>2040</v>
       </c>
       <c r="E27">
         <f t="shared" si="13"/>
-        <v>90000</v>
+        <v>61982.649821833504</v>
       </c>
       <c r="F27">
         <f t="shared" si="14"/>
-        <v>18000</v>
+        <v>6120</v>
       </c>
       <c r="G27">
         <f t="shared" si="15"/>
-        <v>54750</v>
+        <v>48120</v>
       </c>
       <c r="H27">
         <f t="shared" si="16"/>
-        <v>35250</v>
+        <v>13862.649821833504</v>
       </c>
       <c r="I27">
         <f t="shared" si="9"/>
-        <v>620250</v>
+        <v>437962.42306446389</v>
       </c>
       <c r="J27" t="str">
         <f t="shared" si="7"/>
@@ -1823,7 +2968,7 @@
       </c>
       <c r="K27">
         <f t="shared" si="8"/>
-        <v>1762.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
@@ -1832,35 +2977,35 @@
       </c>
       <c r="B28">
         <f t="shared" si="10"/>
-        <v>15750</v>
+        <v>18000</v>
       </c>
       <c r="C28">
         <f t="shared" si="11"/>
-        <v>21000</v>
+        <v>24000</v>
       </c>
       <c r="D28">
         <f t="shared" si="12"/>
-        <v>6000</v>
+        <v>2040</v>
       </c>
       <c r="E28">
         <f t="shared" si="13"/>
-        <v>90000</v>
+        <v>61982.649821833504</v>
       </c>
       <c r="F28">
         <f t="shared" si="14"/>
-        <v>18000</v>
+        <v>6120</v>
       </c>
       <c r="G28">
         <f t="shared" si="15"/>
-        <v>54750</v>
+        <v>48120</v>
       </c>
       <c r="H28">
         <f t="shared" si="16"/>
-        <v>35250</v>
+        <v>13862.649821833504</v>
       </c>
       <c r="I28">
         <f t="shared" si="9"/>
-        <v>655500</v>
+        <v>451825.07288629736</v>
       </c>
       <c r="J28" t="str">
         <f t="shared" si="7"/>
@@ -1868,7 +3013,7 @@
       </c>
       <c r="K28">
         <f t="shared" si="8"/>
-        <v>1762.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
@@ -1877,35 +3022,35 @@
       </c>
       <c r="B29">
         <f t="shared" si="10"/>
-        <v>15750</v>
+        <v>18000</v>
       </c>
       <c r="C29">
         <f t="shared" si="11"/>
-        <v>21000</v>
+        <v>24000</v>
       </c>
       <c r="D29">
         <f t="shared" si="12"/>
-        <v>6000</v>
+        <v>2040</v>
       </c>
       <c r="E29">
         <f t="shared" si="13"/>
-        <v>90000</v>
+        <v>61982.649821833504</v>
       </c>
       <c r="F29">
         <f t="shared" si="14"/>
-        <v>18000</v>
+        <v>6120</v>
       </c>
       <c r="G29">
         <f t="shared" si="15"/>
-        <v>54750</v>
+        <v>48120</v>
       </c>
       <c r="H29">
         <f t="shared" si="16"/>
-        <v>35250</v>
+        <v>13862.649821833504</v>
       </c>
       <c r="I29">
         <f t="shared" si="9"/>
-        <v>690750</v>
+        <v>465687.72270813084</v>
       </c>
       <c r="J29" t="str">
         <f t="shared" si="7"/>
@@ -1913,7 +3058,7 @@
       </c>
       <c r="K29">
         <f t="shared" si="8"/>
-        <v>1762.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
@@ -1922,35 +3067,35 @@
       </c>
       <c r="B30">
         <f t="shared" si="10"/>
-        <v>15750</v>
+        <v>18000</v>
       </c>
       <c r="C30">
         <f t="shared" si="11"/>
-        <v>21000</v>
+        <v>24000</v>
       </c>
       <c r="D30">
         <f t="shared" si="12"/>
-        <v>6000</v>
+        <v>2040</v>
       </c>
       <c r="E30">
         <f t="shared" si="13"/>
-        <v>90000</v>
+        <v>61982.649821833504</v>
       </c>
       <c r="F30">
         <f t="shared" si="14"/>
-        <v>18000</v>
+        <v>6120</v>
       </c>
       <c r="G30">
         <f t="shared" si="15"/>
-        <v>54750</v>
+        <v>48120</v>
       </c>
       <c r="H30">
         <f t="shared" si="16"/>
-        <v>35250</v>
+        <v>13862.649821833504</v>
       </c>
       <c r="I30">
         <f t="shared" si="9"/>
-        <v>726000</v>
+        <v>479550.37252996431</v>
       </c>
       <c r="J30" t="str">
         <f t="shared" si="7"/>
@@ -1958,7 +3103,7 @@
       </c>
       <c r="K30">
         <f t="shared" si="8"/>
-        <v>1762.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
@@ -1967,35 +3112,35 @@
       </c>
       <c r="B31">
         <f t="shared" si="10"/>
-        <v>15750</v>
+        <v>18000</v>
       </c>
       <c r="C31">
         <f t="shared" si="11"/>
-        <v>21000</v>
+        <v>24000</v>
       </c>
       <c r="D31">
         <f t="shared" si="12"/>
-        <v>6000</v>
+        <v>2040</v>
       </c>
       <c r="E31">
         <f t="shared" si="13"/>
-        <v>90000</v>
+        <v>61982.649821833504</v>
       </c>
       <c r="F31">
         <f t="shared" si="14"/>
-        <v>18000</v>
+        <v>6120</v>
       </c>
       <c r="G31">
         <f t="shared" si="15"/>
-        <v>54750</v>
+        <v>48120</v>
       </c>
       <c r="H31">
         <f t="shared" si="16"/>
-        <v>35250</v>
+        <v>13862.649821833504</v>
       </c>
       <c r="I31">
         <f t="shared" si="9"/>
-        <v>761250</v>
+        <v>493413.02235179779</v>
       </c>
       <c r="J31" t="str">
         <f t="shared" si="7"/>
@@ -2003,7 +3148,7 @@
       </c>
       <c r="K31">
         <f t="shared" si="8"/>
-        <v>1762.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
@@ -2012,35 +3157,35 @@
       </c>
       <c r="B32">
         <f t="shared" si="10"/>
-        <v>15750</v>
+        <v>18000</v>
       </c>
       <c r="C32">
         <f t="shared" si="11"/>
-        <v>21000</v>
+        <v>24000</v>
       </c>
       <c r="D32">
         <f t="shared" si="12"/>
-        <v>6000</v>
+        <v>2040</v>
       </c>
       <c r="E32">
         <f t="shared" si="13"/>
-        <v>90000</v>
+        <v>61982.649821833504</v>
       </c>
       <c r="F32">
         <f t="shared" si="14"/>
-        <v>18000</v>
+        <v>6120</v>
       </c>
       <c r="G32">
         <f t="shared" si="15"/>
-        <v>54750</v>
+        <v>48120</v>
       </c>
       <c r="H32">
         <f t="shared" si="16"/>
-        <v>35250</v>
+        <v>13862.649821833504</v>
       </c>
       <c r="I32">
         <f t="shared" si="9"/>
-        <v>796500</v>
+        <v>507275.67217363126</v>
       </c>
       <c r="J32" t="str">
         <f t="shared" si="7"/>
@@ -2048,7 +3193,7 @@
       </c>
       <c r="K32">
         <f t="shared" si="8"/>
-        <v>1762.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
@@ -2057,35 +3202,35 @@
       </c>
       <c r="B33">
         <f t="shared" si="10"/>
-        <v>15750</v>
+        <v>18000</v>
       </c>
       <c r="C33">
         <f t="shared" si="11"/>
-        <v>21000</v>
+        <v>24000</v>
       </c>
       <c r="D33">
         <f t="shared" si="12"/>
-        <v>6000</v>
+        <v>2040</v>
       </c>
       <c r="E33">
         <f t="shared" si="13"/>
-        <v>90000</v>
+        <v>61982.649821833504</v>
       </c>
       <c r="F33">
         <f t="shared" si="14"/>
-        <v>18000</v>
+        <v>6120</v>
       </c>
       <c r="G33">
         <f t="shared" si="15"/>
-        <v>54750</v>
+        <v>48120</v>
       </c>
       <c r="H33">
         <f t="shared" si="16"/>
-        <v>35250</v>
+        <v>13862.649821833504</v>
       </c>
       <c r="I33">
         <f t="shared" si="9"/>
-        <v>831750</v>
+        <v>521138.32199546474</v>
       </c>
       <c r="J33" t="str">
         <f t="shared" si="7"/>
@@ -2093,7 +3238,7 @@
       </c>
       <c r="K33">
         <f t="shared" si="8"/>
-        <v>1762.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
@@ -2102,35 +3247,35 @@
       </c>
       <c r="B34">
         <f t="shared" si="10"/>
-        <v>15750</v>
+        <v>18000</v>
       </c>
       <c r="C34">
         <f t="shared" si="11"/>
-        <v>21000</v>
+        <v>24000</v>
       </c>
       <c r="D34">
         <f t="shared" si="12"/>
-        <v>6000</v>
+        <v>2040</v>
       </c>
       <c r="E34">
         <f t="shared" si="13"/>
-        <v>90000</v>
+        <v>61982.649821833504</v>
       </c>
       <c r="F34">
         <f t="shared" si="14"/>
-        <v>18000</v>
+        <v>6120</v>
       </c>
       <c r="G34">
         <f t="shared" si="15"/>
-        <v>54750</v>
+        <v>48120</v>
       </c>
       <c r="H34">
         <f t="shared" si="16"/>
-        <v>35250</v>
+        <v>13862.649821833504</v>
       </c>
       <c r="I34">
         <f t="shared" si="9"/>
-        <v>867000</v>
+        <v>535000.97181729821</v>
       </c>
       <c r="J34" t="str">
         <f t="shared" si="7"/>
@@ -2138,7 +3283,7 @@
       </c>
       <c r="K34">
         <f t="shared" si="8"/>
-        <v>1762.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
@@ -2147,43 +3292,43 @@
       </c>
       <c r="B35">
         <f>$B$23*(1+$B$7)</f>
-        <v>16537.5</v>
+        <v>21600</v>
       </c>
       <c r="C35">
         <f>C23*(1+$B$7)</f>
-        <v>22050</v>
+        <v>28800</v>
       </c>
       <c r="D35">
         <f>D23*(1+$B$8)</f>
-        <v>6000</v>
+        <v>1734</v>
       </c>
       <c r="E35">
         <f t="shared" si="13"/>
-        <v>90000</v>
+        <v>52685.252348558475</v>
       </c>
       <c r="F35">
         <f t="shared" si="14"/>
-        <v>18000</v>
+        <v>5202</v>
       </c>
       <c r="G35">
         <f t="shared" si="15"/>
-        <v>56587.5</v>
+        <v>55602</v>
       </c>
       <c r="H35">
         <f t="shared" si="16"/>
-        <v>33412.5</v>
+        <v>-2916.7476514415248</v>
       </c>
       <c r="I35">
         <f t="shared" si="9"/>
-        <v>900412.5</v>
+        <v>532084.22416585672</v>
       </c>
       <c r="J35" s="2" t="str">
         <f t="shared" si="7"/>
-        <v>盈利</v>
+        <v>亏损</v>
       </c>
       <c r="K35">
         <f t="shared" si="8"/>
-        <v>1670.625</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
@@ -2192,43 +3337,43 @@
       </c>
       <c r="B36">
         <f t="shared" ref="B36:B46" si="17">$B$23*(1+$B$7)</f>
-        <v>16537.5</v>
+        <v>21600</v>
       </c>
       <c r="C36">
         <f t="shared" ref="C36:C46" si="18">C24*(1+$B$7)</f>
-        <v>22050</v>
+        <v>28800</v>
       </c>
       <c r="D36">
         <f t="shared" ref="D36:D46" si="19">D24*(1+$B$8)</f>
-        <v>6000</v>
+        <v>1734</v>
       </c>
       <c r="E36">
         <f t="shared" si="13"/>
-        <v>90000</v>
+        <v>52685.252348558475</v>
       </c>
       <c r="F36">
         <f t="shared" si="14"/>
-        <v>18000</v>
+        <v>5202</v>
       </c>
       <c r="G36">
         <f t="shared" si="15"/>
-        <v>56587.5</v>
+        <v>55602</v>
       </c>
       <c r="H36">
         <f t="shared" si="16"/>
-        <v>33412.5</v>
+        <v>-2916.7476514415248</v>
       </c>
       <c r="I36">
         <f t="shared" si="9"/>
-        <v>933825</v>
+        <v>529167.47651441523</v>
       </c>
       <c r="J36" s="2" t="str">
         <f t="shared" si="7"/>
-        <v>盈利</v>
+        <v>亏损</v>
       </c>
       <c r="K36">
         <f t="shared" si="8"/>
-        <v>1670.625</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
@@ -2237,43 +3382,43 @@
       </c>
       <c r="B37">
         <f t="shared" si="17"/>
-        <v>16537.5</v>
+        <v>21600</v>
       </c>
       <c r="C37">
         <f t="shared" si="18"/>
-        <v>22050</v>
+        <v>28800</v>
       </c>
       <c r="D37">
         <f t="shared" si="19"/>
-        <v>6000</v>
+        <v>1734</v>
       </c>
       <c r="E37">
         <f t="shared" si="13"/>
-        <v>90000</v>
+        <v>52685.252348558475</v>
       </c>
       <c r="F37">
         <f t="shared" si="14"/>
-        <v>18000</v>
+        <v>5202</v>
       </c>
       <c r="G37">
         <f t="shared" si="15"/>
-        <v>56587.5</v>
+        <v>55602</v>
       </c>
       <c r="H37">
         <f t="shared" si="16"/>
-        <v>33412.5</v>
+        <v>-2916.7476514415248</v>
       </c>
       <c r="I37">
         <f t="shared" si="9"/>
-        <v>967237.5</v>
+        <v>526250.72886297374</v>
       </c>
       <c r="J37" s="2" t="str">
         <f t="shared" si="7"/>
-        <v>盈利</v>
+        <v>亏损</v>
       </c>
       <c r="K37">
         <f t="shared" si="8"/>
-        <v>1670.625</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
@@ -2282,43 +3427,43 @@
       </c>
       <c r="B38">
         <f t="shared" si="17"/>
-        <v>16537.5</v>
+        <v>21600</v>
       </c>
       <c r="C38">
         <f t="shared" si="18"/>
-        <v>22050</v>
+        <v>28800</v>
       </c>
       <c r="D38">
         <f t="shared" si="19"/>
-        <v>6000</v>
+        <v>1734</v>
       </c>
       <c r="E38">
         <f t="shared" si="13"/>
-        <v>90000</v>
+        <v>52685.252348558475</v>
       </c>
       <c r="F38">
         <f t="shared" si="14"/>
-        <v>18000</v>
+        <v>5202</v>
       </c>
       <c r="G38">
         <f t="shared" si="15"/>
-        <v>56587.5</v>
+        <v>55602</v>
       </c>
       <c r="H38">
         <f t="shared" si="16"/>
-        <v>33412.5</v>
+        <v>-2916.7476514415248</v>
       </c>
       <c r="I38">
         <f t="shared" si="9"/>
-        <v>1000650</v>
+        <v>523333.9812115322</v>
       </c>
       <c r="J38" s="2" t="str">
         <f t="shared" si="7"/>
-        <v>盈利</v>
+        <v>亏损</v>
       </c>
       <c r="K38">
         <f t="shared" si="8"/>
-        <v>1670.625</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
@@ -2327,43 +3472,43 @@
       </c>
       <c r="B39">
         <f t="shared" si="17"/>
-        <v>16537.5</v>
+        <v>21600</v>
       </c>
       <c r="C39">
         <f t="shared" si="18"/>
-        <v>22050</v>
+        <v>28800</v>
       </c>
       <c r="D39">
         <f t="shared" si="19"/>
-        <v>6000</v>
+        <v>1734</v>
       </c>
       <c r="E39">
         <f t="shared" si="13"/>
-        <v>90000</v>
+        <v>52685.252348558475</v>
       </c>
       <c r="F39">
         <f t="shared" si="14"/>
-        <v>18000</v>
+        <v>5202</v>
       </c>
       <c r="G39">
         <f t="shared" si="15"/>
-        <v>56587.5</v>
+        <v>55602</v>
       </c>
       <c r="H39">
         <f t="shared" si="16"/>
-        <v>33412.5</v>
+        <v>-2916.7476514415248</v>
       </c>
       <c r="I39">
         <f t="shared" si="9"/>
-        <v>1034062.5</v>
+        <v>520417.23356009065</v>
       </c>
       <c r="J39" s="2" t="str">
         <f t="shared" si="7"/>
-        <v>盈利</v>
+        <v>亏损</v>
       </c>
       <c r="K39">
         <f t="shared" si="8"/>
-        <v>1670.625</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
@@ -2372,43 +3517,43 @@
       </c>
       <c r="B40">
         <f t="shared" si="17"/>
-        <v>16537.5</v>
+        <v>21600</v>
       </c>
       <c r="C40">
         <f t="shared" si="18"/>
-        <v>22050</v>
+        <v>28800</v>
       </c>
       <c r="D40">
         <f t="shared" si="19"/>
-        <v>6000</v>
+        <v>1734</v>
       </c>
       <c r="E40">
         <f t="shared" si="13"/>
-        <v>90000</v>
+        <v>52685.252348558475</v>
       </c>
       <c r="F40">
         <f t="shared" si="14"/>
-        <v>18000</v>
+        <v>5202</v>
       </c>
       <c r="G40">
         <f t="shared" si="15"/>
-        <v>56587.5</v>
+        <v>55602</v>
       </c>
       <c r="H40">
         <f t="shared" si="16"/>
-        <v>33412.5</v>
+        <v>-2916.7476514415248</v>
       </c>
       <c r="I40">
         <f t="shared" si="9"/>
-        <v>1067475</v>
+        <v>517500.48590864911</v>
       </c>
       <c r="J40" s="2" t="str">
         <f t="shared" si="7"/>
-        <v>盈利</v>
+        <v>亏损</v>
       </c>
       <c r="K40">
         <f t="shared" si="8"/>
-        <v>1670.625</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.25">
@@ -2417,43 +3562,43 @@
       </c>
       <c r="B41">
         <f t="shared" si="17"/>
-        <v>16537.5</v>
+        <v>21600</v>
       </c>
       <c r="C41">
         <f t="shared" si="18"/>
-        <v>22050</v>
+        <v>28800</v>
       </c>
       <c r="D41">
         <f t="shared" si="19"/>
-        <v>6000</v>
+        <v>1734</v>
       </c>
       <c r="E41">
         <f t="shared" si="13"/>
-        <v>90000</v>
+        <v>52685.252348558475</v>
       </c>
       <c r="F41">
         <f t="shared" si="14"/>
-        <v>18000</v>
+        <v>5202</v>
       </c>
       <c r="G41">
         <f t="shared" si="15"/>
-        <v>56587.5</v>
+        <v>55602</v>
       </c>
       <c r="H41">
         <f t="shared" si="16"/>
-        <v>33412.5</v>
+        <v>-2916.7476514415248</v>
       </c>
       <c r="I41">
         <f t="shared" si="9"/>
-        <v>1100887.5</v>
+        <v>514583.73825720756</v>
       </c>
       <c r="J41" s="2" t="str">
         <f t="shared" si="7"/>
-        <v>盈利</v>
+        <v>亏损</v>
       </c>
       <c r="K41">
         <f t="shared" si="8"/>
-        <v>1670.625</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.25">
@@ -2462,43 +3607,43 @@
       </c>
       <c r="B42">
         <f t="shared" si="17"/>
-        <v>16537.5</v>
+        <v>21600</v>
       </c>
       <c r="C42">
         <f t="shared" si="18"/>
-        <v>22050</v>
+        <v>28800</v>
       </c>
       <c r="D42">
         <f t="shared" si="19"/>
-        <v>6000</v>
+        <v>1734</v>
       </c>
       <c r="E42">
         <f t="shared" si="13"/>
-        <v>90000</v>
+        <v>52685.252348558475</v>
       </c>
       <c r="F42">
         <f t="shared" si="14"/>
-        <v>18000</v>
+        <v>5202</v>
       </c>
       <c r="G42">
         <f t="shared" si="15"/>
-        <v>56587.5</v>
+        <v>55602</v>
       </c>
       <c r="H42">
         <f t="shared" si="16"/>
-        <v>33412.5</v>
+        <v>-2916.7476514415248</v>
       </c>
       <c r="I42">
         <f t="shared" si="9"/>
-        <v>1134300</v>
+        <v>511666.99060576601</v>
       </c>
       <c r="J42" s="2" t="str">
         <f t="shared" si="7"/>
-        <v>盈利</v>
+        <v>亏损</v>
       </c>
       <c r="K42">
         <f t="shared" si="8"/>
-        <v>1670.625</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.25">
@@ -2507,43 +3652,43 @@
       </c>
       <c r="B43">
         <f t="shared" si="17"/>
-        <v>16537.5</v>
+        <v>21600</v>
       </c>
       <c r="C43">
         <f t="shared" si="18"/>
-        <v>22050</v>
+        <v>28800</v>
       </c>
       <c r="D43">
         <f t="shared" si="19"/>
-        <v>6000</v>
+        <v>1734</v>
       </c>
       <c r="E43">
         <f t="shared" si="13"/>
-        <v>90000</v>
+        <v>52685.252348558475</v>
       </c>
       <c r="F43">
         <f t="shared" si="14"/>
-        <v>18000</v>
+        <v>5202</v>
       </c>
       <c r="G43">
         <f t="shared" si="15"/>
-        <v>56587.5</v>
+        <v>55602</v>
       </c>
       <c r="H43">
         <f t="shared" si="16"/>
-        <v>33412.5</v>
+        <v>-2916.7476514415248</v>
       </c>
       <c r="I43">
         <f t="shared" si="9"/>
-        <v>1167712.5</v>
+        <v>508750.24295432447</v>
       </c>
       <c r="J43" s="2" t="str">
         <f t="shared" si="7"/>
-        <v>盈利</v>
+        <v>亏损</v>
       </c>
       <c r="K43">
         <f t="shared" si="8"/>
-        <v>1670.625</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.25">
@@ -2552,43 +3697,43 @@
       </c>
       <c r="B44">
         <f t="shared" si="17"/>
-        <v>16537.5</v>
+        <v>21600</v>
       </c>
       <c r="C44">
         <f t="shared" si="18"/>
-        <v>22050</v>
+        <v>28800</v>
       </c>
       <c r="D44">
         <f t="shared" si="19"/>
-        <v>6000</v>
+        <v>1734</v>
       </c>
       <c r="E44">
         <f t="shared" si="13"/>
-        <v>90000</v>
+        <v>52685.252348558475</v>
       </c>
       <c r="F44">
         <f t="shared" si="14"/>
-        <v>18000</v>
+        <v>5202</v>
       </c>
       <c r="G44">
         <f t="shared" si="15"/>
-        <v>56587.5</v>
+        <v>55602</v>
       </c>
       <c r="H44">
         <f t="shared" si="16"/>
-        <v>33412.5</v>
+        <v>-2916.7476514415248</v>
       </c>
       <c r="I44">
         <f t="shared" si="9"/>
-        <v>1201125</v>
+        <v>505833.49530288292</v>
       </c>
       <c r="J44" s="2" t="str">
         <f t="shared" si="7"/>
-        <v>盈利</v>
+        <v>亏损</v>
       </c>
       <c r="K44">
         <f t="shared" si="8"/>
-        <v>1670.625</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.25">
@@ -2597,43 +3742,43 @@
       </c>
       <c r="B45">
         <f t="shared" si="17"/>
-        <v>16537.5</v>
+        <v>21600</v>
       </c>
       <c r="C45">
         <f t="shared" si="18"/>
-        <v>22050</v>
+        <v>28800</v>
       </c>
       <c r="D45">
         <f t="shared" si="19"/>
-        <v>6000</v>
+        <v>1734</v>
       </c>
       <c r="E45">
         <f t="shared" si="13"/>
-        <v>90000</v>
+        <v>52685.252348558475</v>
       </c>
       <c r="F45">
         <f t="shared" si="14"/>
-        <v>18000</v>
+        <v>5202</v>
       </c>
       <c r="G45">
         <f t="shared" si="15"/>
-        <v>56587.5</v>
+        <v>55602</v>
       </c>
       <c r="H45">
         <f t="shared" si="16"/>
-        <v>33412.5</v>
+        <v>-2916.7476514415248</v>
       </c>
       <c r="I45">
         <f t="shared" si="9"/>
-        <v>1234537.5</v>
+        <v>502916.74765144137</v>
       </c>
       <c r="J45" s="2" t="str">
         <f t="shared" si="7"/>
-        <v>盈利</v>
+        <v>亏损</v>
       </c>
       <c r="K45">
         <f t="shared" si="8"/>
-        <v>1670.625</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.25">
@@ -2642,47 +3787,47 @@
       </c>
       <c r="B46">
         <f t="shared" si="17"/>
-        <v>16537.5</v>
+        <v>21600</v>
       </c>
       <c r="C46">
         <f t="shared" si="18"/>
-        <v>22050</v>
+        <v>28800</v>
       </c>
       <c r="D46">
         <f t="shared" si="19"/>
-        <v>6000</v>
+        <v>1734</v>
       </c>
       <c r="E46">
         <f t="shared" si="13"/>
-        <v>90000</v>
+        <v>52685.252348558475</v>
       </c>
       <c r="F46">
         <f t="shared" si="14"/>
-        <v>18000</v>
+        <v>5202</v>
       </c>
       <c r="G46">
         <f t="shared" si="15"/>
-        <v>56587.5</v>
+        <v>55602</v>
       </c>
       <c r="H46">
         <f t="shared" si="16"/>
-        <v>33412.5</v>
+        <v>-2916.7476514415248</v>
       </c>
       <c r="I46">
         <f t="shared" si="9"/>
-        <v>1267950</v>
+        <v>499999.99999999983</v>
       </c>
       <c r="J46" s="2" t="str">
         <f t="shared" si="7"/>
-        <v>盈利</v>
+        <v>亏损</v>
       </c>
       <c r="K46">
         <f t="shared" si="8"/>
-        <v>1670.625</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
-  <scenarios current="2" show="1" sqref="I46">
+  <scenarios current="2" show="2" sqref="I46">
     <scenario name="基准情景" locked="1" count="4" user="Administrator" comment="创建者 Administrator 日期 2026/9/16">
       <inputCells r="B4" val="13"/>
       <inputCells r="B5" val="150"/>
@@ -2705,4 +3850,147 @@
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>15</v>
+      </c>
+      <c r="B2">
+        <v>100</v>
+      </c>
+      <c r="C2">
+        <f>((B3-B2)/((B2+B3)/2))/((A3-A2)/((A2+A3)/2))</f>
+        <v>-5.8000000000000007</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>14</v>
+      </c>
+      <c r="B3">
+        <v>150</v>
+      </c>
+      <c r="C3">
+        <f t="shared" ref="C3:C11" si="0">((B4-B3)/((B3+B4)/2))/((A4-A3)/((A3+A4)/2))</f>
+        <v>-3.8571428571428572</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>13</v>
+      </c>
+      <c r="B4">
+        <v>200</v>
+      </c>
+      <c r="C4">
+        <f t="shared" si="0"/>
+        <v>-2.7777777777777777</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>12</v>
+      </c>
+      <c r="B5">
+        <v>250</v>
+      </c>
+      <c r="C5">
+        <f t="shared" si="0"/>
+        <v>-2.0909090909090908</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>11</v>
+      </c>
+      <c r="B6">
+        <v>300</v>
+      </c>
+      <c r="C6">
+        <f t="shared" si="0"/>
+        <v>-1.6153846153846156</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>10</v>
+      </c>
+      <c r="B7">
+        <v>350</v>
+      </c>
+      <c r="C7">
+        <f t="shared" si="0"/>
+        <v>-1.2666666666666668</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>9</v>
+      </c>
+      <c r="B8">
+        <v>400</v>
+      </c>
+      <c r="C8">
+        <f t="shared" si="0"/>
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>450</v>
+      </c>
+      <c r="C9">
+        <f t="shared" si="0"/>
+        <v>-0.78947368421052633</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>7</v>
+      </c>
+      <c r="B10">
+        <v>500</v>
+      </c>
+      <c r="C10">
+        <f t="shared" si="0"/>
+        <v>-0.61904761904761896</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>6</v>
+      </c>
+      <c r="B11">
+        <v>550</v>
+      </c>
+      <c r="C11">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs: daily log Sep 18
</commit_message>
<xml_diff>
--- a/tea_shop_model.xlsx
+++ b/tea_shop_model.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="9192" windowHeight="2988" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="9192" windowHeight="2988" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="方案摘要" sheetId="2" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="80">
   <si>
     <t>初始月租金</t>
     <phoneticPr fontId="2" type="noConversion"/>
@@ -274,6 +274,26 @@
   </si>
   <si>
     <t>PED</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>盈亏平衡分析</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>单杯边际效应（卖出一杯奶茶赚到的"毛利"）</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>月盈亏平衡销量（每个月至少要卖多少杯才能不亏钱</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>（折算到一天要卖多少杯)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>三年内亏损数量</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -535,6 +555,37 @@
   </mc:AlternateContent>
   <c:chart>
     <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Lower Price Drives Higher Demand</a:t>
+            </a:r>
+          </a:p>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
       <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
@@ -567,7 +618,17 @@
     </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
-      <c:layout/>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="4.7614489190043137E-2"/>
+          <c:y val="0.20782508630609897"/>
+          <c:w val="0.92489246353145083"/>
+          <c:h val="0.71853368731670342"/>
+        </c:manualLayout>
+      </c:layout>
       <c:scatterChart>
         <c:scatterStyle val="lineMarker"/>
         <c:varyColors val="0"/>
@@ -601,6 +662,270 @@
               <a:effectLst/>
             </c:spPr>
           </c:marker>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:marker>
+              <c:symbol val="circle"/>
+              <c:size val="5"/>
+              <c:spPr>
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:ln w="9525">
+                  <a:solidFill>
+                    <a:schemeClr val="accent1"/>
+                  </a:solidFill>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+            </c:marker>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:ln w="28575" cap="rnd">
+                <a:solidFill>
+                  <a:srgbClr val="FF0000"/>
+                </a:solidFill>
+                <a:round/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000002-A2B5-4BAC-97D0-44981B88D339}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:marker>
+              <c:symbol val="circle"/>
+              <c:size val="5"/>
+              <c:spPr>
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:ln w="9525">
+                  <a:solidFill>
+                    <a:schemeClr val="accent1"/>
+                  </a:solidFill>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+            </c:marker>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:ln w="28575" cap="rnd">
+                <a:solidFill>
+                  <a:srgbClr val="FF0000"/>
+                </a:solidFill>
+                <a:round/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-A2B5-4BAC-97D0-44981B88D339}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="3"/>
+            <c:marker>
+              <c:symbol val="circle"/>
+              <c:size val="5"/>
+              <c:spPr>
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:ln w="9525">
+                  <a:solidFill>
+                    <a:schemeClr val="accent1"/>
+                  </a:solidFill>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+            </c:marker>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:ln w="28575" cap="rnd">
+                <a:solidFill>
+                  <a:srgbClr val="FF0000"/>
+                </a:solidFill>
+                <a:round/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-A2B5-4BAC-97D0-44981B88D339}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="5"/>
+            <c:marker>
+              <c:symbol val="circle"/>
+              <c:size val="5"/>
+              <c:spPr>
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:ln w="9525">
+                  <a:solidFill>
+                    <a:schemeClr val="accent1"/>
+                  </a:solidFill>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+            </c:marker>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:round/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000007-A2B5-4BAC-97D0-44981B88D339}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="6"/>
+            <c:marker>
+              <c:symbol val="circle"/>
+              <c:size val="5"/>
+              <c:spPr>
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:ln w="9525">
+                  <a:solidFill>
+                    <a:schemeClr val="accent1"/>
+                  </a:solidFill>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+            </c:marker>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:ln w="28575" cap="rnd">
+                <a:solidFill>
+                  <a:srgbClr val="0070C0"/>
+                </a:solidFill>
+                <a:round/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000008-A2B5-4BAC-97D0-44981B88D339}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="7"/>
+            <c:marker>
+              <c:symbol val="circle"/>
+              <c:size val="5"/>
+              <c:spPr>
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:ln w="9525">
+                  <a:solidFill>
+                    <a:schemeClr val="accent1"/>
+                  </a:solidFill>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+            </c:marker>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:ln w="28575" cap="rnd">
+                <a:solidFill>
+                  <a:srgbClr val="0070C0"/>
+                </a:solidFill>
+                <a:round/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000005-A2B5-4BAC-97D0-44981B88D339}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="8"/>
+            <c:marker>
+              <c:symbol val="circle"/>
+              <c:size val="5"/>
+              <c:spPr>
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:ln w="9525">
+                  <a:solidFill>
+                    <a:schemeClr val="accent1"/>
+                  </a:solidFill>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+            </c:marker>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:ln w="28575" cap="rnd">
+                <a:solidFill>
+                  <a:srgbClr val="0070C0"/>
+                </a:solidFill>
+                <a:round/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000006-A2B5-4BAC-97D0-44981B88D339}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="9"/>
+            <c:marker>
+              <c:symbol val="circle"/>
+              <c:size val="5"/>
+              <c:spPr>
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:ln w="9525">
+                  <a:solidFill>
+                    <a:schemeClr val="accent1"/>
+                  </a:solidFill>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+            </c:marker>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:ln w="28575" cap="rnd">
+                <a:solidFill>
+                  <a:srgbClr val="0070C0"/>
+                </a:solidFill>
+                <a:round/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000004-A2B5-4BAC-97D0-44981B88D339}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
           <c:xVal>
             <c:numRef>
               <c:f>Demand_Curve!$B$2:$B$11</c:f>
@@ -718,37 +1043,6 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
-        <c:title>
-          <c:layout/>
-          <c:overlay val="0"/>
-          <c:spPr>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="65000"/>
-                      <a:lumOff val="35000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="zh-CN"/>
-            </a:p>
-          </c:txPr>
-        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -797,20 +1091,6 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -854,7 +1134,7 @@
       </c:valAx>
       <c:spPr>
         <a:noFill/>
-        <a:ln>
+        <a:ln w="25400">
           <a:noFill/>
         </a:ln>
         <a:effectLst/>
@@ -1459,15 +1739,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>53340</xdr:colOff>
+      <xdr:colOff>60960</xdr:colOff>
       <xdr:row>10</xdr:row>
-      <xdr:rowOff>87630</xdr:rowOff>
+      <xdr:rowOff>125730</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
+      <xdr:col>18</xdr:col>
       <xdr:colOff>358140</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>26670</xdr:rowOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>106680</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2099,14 +2379,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K46"/>
+  <dimension ref="A1:M46"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.109375" customWidth="1"/>
     <col min="6" max="6" width="11" customWidth="1"/>
+    <col min="12" max="12" width="14.33203125" customWidth="1"/>
+    <col min="13" max="13" width="40.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2114,7 +2396,7 @@
         <v>15000</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -2122,7 +2404,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -2130,23 +2412,23 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
       <c r="B4">
-        <v>30.383651873447796</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
       <c r="B5">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -2155,23 +2437,23 @@
         <v>35000</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>6</v>
       </c>
       <c r="B7" s="1">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>7</v>
       </c>
       <c r="B8" s="1">
-        <v>-0.15</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+        <v>-0.05</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -2205,8 +2487,11 @@
       <c r="K10" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L10" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>17</v>
       </c>
@@ -2220,27 +2505,27 @@
       </c>
       <c r="D11">
         <f>$B$5*30</f>
-        <v>2400</v>
+        <v>4500</v>
       </c>
       <c r="E11">
         <f>$B$4*D11</f>
-        <v>72920.764496274714</v>
+        <v>58500</v>
       </c>
       <c r="F11">
         <f>$B$3*D11</f>
-        <v>7200</v>
+        <v>13500</v>
       </c>
       <c r="G11">
         <f>B11+C11+F11</f>
-        <v>42200</v>
+        <v>48500</v>
       </c>
       <c r="H11">
         <f>E11-G11</f>
-        <v>30720.764496274714</v>
+        <v>10000</v>
       </c>
       <c r="I11">
         <f>H11</f>
-        <v>30720.764496274714</v>
+        <v>10000</v>
       </c>
       <c r="J11" t="str">
         <f>IF(H11&gt;50000,"优秀",IF(H11&gt;0,"盈利",IF(H11=0,"保本","亏损")))</f>
@@ -2248,10 +2533,17 @@
       </c>
       <c r="K11">
         <f>IF(H11&lt;0,0,IF(D11&gt;4500,H11*0.05,IF(D11&gt;3500,H11*0.02,0)))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+        <v>200</v>
+      </c>
+      <c r="L11">
+        <f>B4-B3</f>
+        <v>10</v>
+      </c>
+      <c r="M11" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>18</v>
       </c>
@@ -2265,27 +2557,27 @@
       </c>
       <c r="D12">
         <f t="shared" ref="D12:D22" si="2">$B$5*30</f>
-        <v>2400</v>
+        <v>4500</v>
       </c>
       <c r="E12">
         <f t="shared" ref="E12:E22" si="3">$B$4*D12</f>
-        <v>72920.764496274714</v>
+        <v>58500</v>
       </c>
       <c r="F12">
         <f t="shared" ref="F12:F22" si="4">$B$3*D12</f>
-        <v>7200</v>
+        <v>13500</v>
       </c>
       <c r="G12">
         <f t="shared" ref="G12:G22" si="5">B12+C12+F12</f>
-        <v>42200</v>
+        <v>48500</v>
       </c>
       <c r="H12">
         <f t="shared" ref="H12:H22" si="6">E12-G12</f>
-        <v>30720.764496274714</v>
+        <v>10000</v>
       </c>
       <c r="I12">
         <f>H12+I11</f>
-        <v>61441.528992549429</v>
+        <v>20000</v>
       </c>
       <c r="J12" t="str">
         <f t="shared" ref="J12:J46" si="7">IF(H12&gt;50000,"优秀",IF(H12&gt;0,"盈利",IF(H12=0,"保本","亏损")))</f>
@@ -2293,10 +2585,17 @@
       </c>
       <c r="K12">
         <f t="shared" ref="K12:K46" si="8">IF(H12&lt;0,0,IF(D12&gt;4500,H12*0.05,IF(D12&gt;3500,H12*0.02,0)))</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+        <v>200</v>
+      </c>
+      <c r="L12">
+        <f>B6/L11</f>
+        <v>3500</v>
+      </c>
+      <c r="M12" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>19</v>
       </c>
@@ -2310,27 +2609,27 @@
       </c>
       <c r="D13">
         <f t="shared" si="2"/>
-        <v>2400</v>
+        <v>4500</v>
       </c>
       <c r="E13">
         <f t="shared" si="3"/>
-        <v>72920.764496274714</v>
+        <v>58500</v>
       </c>
       <c r="F13">
         <f t="shared" si="4"/>
-        <v>7200</v>
+        <v>13500</v>
       </c>
       <c r="G13">
         <f t="shared" si="5"/>
-        <v>42200</v>
+        <v>48500</v>
       </c>
       <c r="H13">
         <f t="shared" si="6"/>
-        <v>30720.764496274714</v>
+        <v>10000</v>
       </c>
       <c r="I13">
         <f t="shared" ref="I13:I46" si="9">H13+I12</f>
-        <v>92162.293488824143</v>
+        <v>30000</v>
       </c>
       <c r="J13" t="str">
         <f t="shared" si="7"/>
@@ -2338,10 +2637,17 @@
       </c>
       <c r="K13">
         <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+        <v>200</v>
+      </c>
+      <c r="L13">
+        <f>L12/30</f>
+        <v>116.66666666666667</v>
+      </c>
+      <c r="M13" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>20</v>
       </c>
@@ -2355,27 +2661,27 @@
       </c>
       <c r="D14">
         <f t="shared" si="2"/>
-        <v>2400</v>
+        <v>4500</v>
       </c>
       <c r="E14">
         <f t="shared" si="3"/>
-        <v>72920.764496274714</v>
+        <v>58500</v>
       </c>
       <c r="F14">
         <f t="shared" si="4"/>
-        <v>7200</v>
+        <v>13500</v>
       </c>
       <c r="G14">
         <f t="shared" si="5"/>
-        <v>42200</v>
+        <v>48500</v>
       </c>
       <c r="H14">
         <f t="shared" si="6"/>
-        <v>30720.764496274714</v>
+        <v>10000</v>
       </c>
       <c r="I14">
         <f t="shared" si="9"/>
-        <v>122883.05798509886</v>
+        <v>40000</v>
       </c>
       <c r="J14" t="str">
         <f t="shared" si="7"/>
@@ -2383,10 +2689,17 @@
       </c>
       <c r="K14">
         <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+        <v>200</v>
+      </c>
+      <c r="L14">
+        <f>COUNTIF(J11:J46,"亏损")</f>
+        <v>12</v>
+      </c>
+      <c r="M14" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>21</v>
       </c>
@@ -2400,27 +2713,27 @@
       </c>
       <c r="D15">
         <f t="shared" si="2"/>
-        <v>2400</v>
+        <v>4500</v>
       </c>
       <c r="E15">
         <f t="shared" si="3"/>
-        <v>72920.764496274714</v>
+        <v>58500</v>
       </c>
       <c r="F15">
         <f t="shared" si="4"/>
-        <v>7200</v>
+        <v>13500</v>
       </c>
       <c r="G15">
         <f t="shared" si="5"/>
-        <v>42200</v>
+        <v>48500</v>
       </c>
       <c r="H15">
         <f t="shared" si="6"/>
-        <v>30720.764496274714</v>
+        <v>10000</v>
       </c>
       <c r="I15">
         <f t="shared" si="9"/>
-        <v>153603.82248137356</v>
+        <v>50000</v>
       </c>
       <c r="J15" t="str">
         <f t="shared" si="7"/>
@@ -2428,10 +2741,10 @@
       </c>
       <c r="K15">
         <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>22</v>
       </c>
@@ -2445,27 +2758,27 @@
       </c>
       <c r="D16">
         <f t="shared" si="2"/>
-        <v>2400</v>
+        <v>4500</v>
       </c>
       <c r="E16">
         <f t="shared" si="3"/>
-        <v>72920.764496274714</v>
+        <v>58500</v>
       </c>
       <c r="F16">
         <f t="shared" si="4"/>
-        <v>7200</v>
+        <v>13500</v>
       </c>
       <c r="G16">
         <f t="shared" si="5"/>
-        <v>42200</v>
+        <v>48500</v>
       </c>
       <c r="H16">
         <f t="shared" si="6"/>
-        <v>30720.764496274714</v>
+        <v>10000</v>
       </c>
       <c r="I16">
         <f t="shared" si="9"/>
-        <v>184324.58697764826</v>
+        <v>60000</v>
       </c>
       <c r="J16" t="str">
         <f t="shared" si="7"/>
@@ -2473,7 +2786,7 @@
       </c>
       <c r="K16">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>200</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
@@ -2490,27 +2803,27 @@
       </c>
       <c r="D17">
         <f t="shared" si="2"/>
-        <v>2400</v>
+        <v>4500</v>
       </c>
       <c r="E17">
         <f t="shared" si="3"/>
-        <v>72920.764496274714</v>
+        <v>58500</v>
       </c>
       <c r="F17">
         <f t="shared" si="4"/>
-        <v>7200</v>
+        <v>13500</v>
       </c>
       <c r="G17">
         <f t="shared" si="5"/>
-        <v>42200</v>
+        <v>48500</v>
       </c>
       <c r="H17">
         <f t="shared" si="6"/>
-        <v>30720.764496274714</v>
+        <v>10000</v>
       </c>
       <c r="I17">
         <f t="shared" si="9"/>
-        <v>215045.35147392296</v>
+        <v>70000</v>
       </c>
       <c r="J17" t="str">
         <f t="shared" si="7"/>
@@ -2518,7 +2831,7 @@
       </c>
       <c r="K17">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>200</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
@@ -2535,27 +2848,27 @@
       </c>
       <c r="D18">
         <f t="shared" si="2"/>
-        <v>2400</v>
+        <v>4500</v>
       </c>
       <c r="E18">
         <f t="shared" si="3"/>
-        <v>72920.764496274714</v>
+        <v>58500</v>
       </c>
       <c r="F18">
         <f t="shared" si="4"/>
-        <v>7200</v>
+        <v>13500</v>
       </c>
       <c r="G18">
         <f t="shared" si="5"/>
-        <v>42200</v>
+        <v>48500</v>
       </c>
       <c r="H18">
         <f t="shared" si="6"/>
-        <v>30720.764496274714</v>
+        <v>10000</v>
       </c>
       <c r="I18">
         <f t="shared" si="9"/>
-        <v>245766.11597019766</v>
+        <v>80000</v>
       </c>
       <c r="J18" t="str">
         <f t="shared" si="7"/>
@@ -2563,7 +2876,7 @@
       </c>
       <c r="K18">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>200</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
@@ -2580,27 +2893,27 @@
       </c>
       <c r="D19">
         <f t="shared" si="2"/>
-        <v>2400</v>
+        <v>4500</v>
       </c>
       <c r="E19">
         <f t="shared" si="3"/>
-        <v>72920.764496274714</v>
+        <v>58500</v>
       </c>
       <c r="F19">
         <f t="shared" si="4"/>
-        <v>7200</v>
+        <v>13500</v>
       </c>
       <c r="G19">
         <f t="shared" si="5"/>
-        <v>42200</v>
+        <v>48500</v>
       </c>
       <c r="H19">
         <f t="shared" si="6"/>
-        <v>30720.764496274714</v>
+        <v>10000</v>
       </c>
       <c r="I19">
         <f t="shared" si="9"/>
-        <v>276486.88046647236</v>
+        <v>90000</v>
       </c>
       <c r="J19" t="str">
         <f t="shared" si="7"/>
@@ -2608,7 +2921,7 @@
       </c>
       <c r="K19">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>200</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
@@ -2625,27 +2938,27 @@
       </c>
       <c r="D20">
         <f t="shared" si="2"/>
-        <v>2400</v>
+        <v>4500</v>
       </c>
       <c r="E20">
         <f t="shared" si="3"/>
-        <v>72920.764496274714</v>
+        <v>58500</v>
       </c>
       <c r="F20">
         <f t="shared" si="4"/>
-        <v>7200</v>
+        <v>13500</v>
       </c>
       <c r="G20">
         <f t="shared" si="5"/>
-        <v>42200</v>
+        <v>48500</v>
       </c>
       <c r="H20">
         <f t="shared" si="6"/>
-        <v>30720.764496274714</v>
+        <v>10000</v>
       </c>
       <c r="I20">
         <f t="shared" si="9"/>
-        <v>307207.64496274706</v>
+        <v>100000</v>
       </c>
       <c r="J20" t="str">
         <f t="shared" si="7"/>
@@ -2653,7 +2966,7 @@
       </c>
       <c r="K20">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>200</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
@@ -2670,27 +2983,27 @@
       </c>
       <c r="D21">
         <f t="shared" si="2"/>
-        <v>2400</v>
+        <v>4500</v>
       </c>
       <c r="E21">
         <f t="shared" si="3"/>
-        <v>72920.764496274714</v>
+        <v>58500</v>
       </c>
       <c r="F21">
         <f t="shared" si="4"/>
-        <v>7200</v>
+        <v>13500</v>
       </c>
       <c r="G21">
         <f t="shared" si="5"/>
-        <v>42200</v>
+        <v>48500</v>
       </c>
       <c r="H21">
         <f t="shared" si="6"/>
-        <v>30720.764496274714</v>
+        <v>10000</v>
       </c>
       <c r="I21">
         <f t="shared" si="9"/>
-        <v>337928.40945902176</v>
+        <v>110000</v>
       </c>
       <c r="J21" t="str">
         <f t="shared" si="7"/>
@@ -2698,7 +3011,7 @@
       </c>
       <c r="K21">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>200</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
@@ -2715,27 +3028,27 @@
       </c>
       <c r="D22">
         <f t="shared" si="2"/>
-        <v>2400</v>
+        <v>4500</v>
       </c>
       <c r="E22">
         <f t="shared" si="3"/>
-        <v>72920.764496274714</v>
+        <v>58500</v>
       </c>
       <c r="F22">
         <f t="shared" si="4"/>
-        <v>7200</v>
+        <v>13500</v>
       </c>
       <c r="G22">
         <f t="shared" si="5"/>
-        <v>42200</v>
+        <v>48500</v>
       </c>
       <c r="H22">
         <f t="shared" si="6"/>
-        <v>30720.764496274714</v>
+        <v>10000</v>
       </c>
       <c r="I22">
         <f t="shared" si="9"/>
-        <v>368649.17395529646</v>
+        <v>120000</v>
       </c>
       <c r="J22" t="str">
         <f t="shared" si="7"/>
@@ -2743,7 +3056,7 @@
       </c>
       <c r="K22">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>200</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
@@ -2752,35 +3065,35 @@
       </c>
       <c r="B23">
         <f>$B$1*(1+$B$7)</f>
-        <v>18000</v>
+        <v>17250</v>
       </c>
       <c r="C23">
         <f>$B$2*(1+$B$7)</f>
-        <v>24000</v>
+        <v>23000</v>
       </c>
       <c r="D23">
         <f>$B$5*30*(1+$B$8)</f>
-        <v>2040</v>
+        <v>4275</v>
       </c>
       <c r="E23">
         <f>$B$4*D23</f>
-        <v>61982.649821833504</v>
+        <v>55575</v>
       </c>
       <c r="F23">
         <f>$B$3*D23</f>
-        <v>6120</v>
+        <v>12825</v>
       </c>
       <c r="G23">
         <f>B23+C23+F23</f>
-        <v>48120</v>
+        <v>53075</v>
       </c>
       <c r="H23">
         <f>E23-G23</f>
-        <v>13862.649821833504</v>
+        <v>2500</v>
       </c>
       <c r="I23">
         <f t="shared" si="9"/>
-        <v>382511.82377712999</v>
+        <v>122500</v>
       </c>
       <c r="J23" t="str">
         <f t="shared" si="7"/>
@@ -2788,7 +3101,7 @@
       </c>
       <c r="K23">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
@@ -2797,35 +3110,35 @@
       </c>
       <c r="B24">
         <f t="shared" ref="B24:B34" si="10">$B$1*(1+$B$7)</f>
-        <v>18000</v>
+        <v>17250</v>
       </c>
       <c r="C24">
         <f t="shared" ref="C24:C34" si="11">$B$2*(1+$B$7)</f>
-        <v>24000</v>
+        <v>23000</v>
       </c>
       <c r="D24">
         <f t="shared" ref="D24:D34" si="12">$B$5*30*(1+$B$8)</f>
-        <v>2040</v>
+        <v>4275</v>
       </c>
       <c r="E24">
         <f t="shared" ref="E24:E46" si="13">$B$4*D24</f>
-        <v>61982.649821833504</v>
+        <v>55575</v>
       </c>
       <c r="F24">
         <f t="shared" ref="F24:F46" si="14">$B$3*D24</f>
-        <v>6120</v>
+        <v>12825</v>
       </c>
       <c r="G24">
         <f t="shared" ref="G24:G46" si="15">B24+C24+F24</f>
-        <v>48120</v>
+        <v>53075</v>
       </c>
       <c r="H24">
         <f t="shared" ref="H24:H46" si="16">E24-G24</f>
-        <v>13862.649821833504</v>
+        <v>2500</v>
       </c>
       <c r="I24">
         <f t="shared" si="9"/>
-        <v>396374.47359896346</v>
+        <v>125000</v>
       </c>
       <c r="J24" t="str">
         <f t="shared" si="7"/>
@@ -2833,7 +3146,7 @@
       </c>
       <c r="K24">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
@@ -2842,35 +3155,35 @@
       </c>
       <c r="B25">
         <f t="shared" si="10"/>
-        <v>18000</v>
+        <v>17250</v>
       </c>
       <c r="C25">
         <f t="shared" si="11"/>
-        <v>24000</v>
+        <v>23000</v>
       </c>
       <c r="D25">
         <f t="shared" si="12"/>
-        <v>2040</v>
+        <v>4275</v>
       </c>
       <c r="E25">
         <f t="shared" si="13"/>
-        <v>61982.649821833504</v>
+        <v>55575</v>
       </c>
       <c r="F25">
         <f t="shared" si="14"/>
-        <v>6120</v>
+        <v>12825</v>
       </c>
       <c r="G25">
         <f t="shared" si="15"/>
-        <v>48120</v>
+        <v>53075</v>
       </c>
       <c r="H25">
         <f t="shared" si="16"/>
-        <v>13862.649821833504</v>
+        <v>2500</v>
       </c>
       <c r="I25">
         <f t="shared" si="9"/>
-        <v>410237.12342079694</v>
+        <v>127500</v>
       </c>
       <c r="J25" t="str">
         <f t="shared" si="7"/>
@@ -2878,7 +3191,7 @@
       </c>
       <c r="K25">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
@@ -2887,35 +3200,35 @@
       </c>
       <c r="B26">
         <f t="shared" si="10"/>
-        <v>18000</v>
+        <v>17250</v>
       </c>
       <c r="C26">
         <f t="shared" si="11"/>
-        <v>24000</v>
+        <v>23000</v>
       </c>
       <c r="D26">
         <f t="shared" si="12"/>
-        <v>2040</v>
+        <v>4275</v>
       </c>
       <c r="E26">
         <f t="shared" si="13"/>
-        <v>61982.649821833504</v>
+        <v>55575</v>
       </c>
       <c r="F26">
         <f t="shared" si="14"/>
-        <v>6120</v>
+        <v>12825</v>
       </c>
       <c r="G26">
         <f t="shared" si="15"/>
-        <v>48120</v>
+        <v>53075</v>
       </c>
       <c r="H26">
         <f t="shared" si="16"/>
-        <v>13862.649821833504</v>
+        <v>2500</v>
       </c>
       <c r="I26">
         <f t="shared" si="9"/>
-        <v>424099.77324263041</v>
+        <v>130000</v>
       </c>
       <c r="J26" t="str">
         <f t="shared" si="7"/>
@@ -2923,7 +3236,7 @@
       </c>
       <c r="K26">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
@@ -2932,35 +3245,35 @@
       </c>
       <c r="B27">
         <f t="shared" si="10"/>
-        <v>18000</v>
+        <v>17250</v>
       </c>
       <c r="C27">
         <f t="shared" si="11"/>
-        <v>24000</v>
+        <v>23000</v>
       </c>
       <c r="D27">
         <f t="shared" si="12"/>
-        <v>2040</v>
+        <v>4275</v>
       </c>
       <c r="E27">
         <f t="shared" si="13"/>
-        <v>61982.649821833504</v>
+        <v>55575</v>
       </c>
       <c r="F27">
         <f t="shared" si="14"/>
-        <v>6120</v>
+        <v>12825</v>
       </c>
       <c r="G27">
         <f t="shared" si="15"/>
-        <v>48120</v>
+        <v>53075</v>
       </c>
       <c r="H27">
         <f t="shared" si="16"/>
-        <v>13862.649821833504</v>
+        <v>2500</v>
       </c>
       <c r="I27">
         <f t="shared" si="9"/>
-        <v>437962.42306446389</v>
+        <v>132500</v>
       </c>
       <c r="J27" t="str">
         <f t="shared" si="7"/>
@@ -2968,7 +3281,7 @@
       </c>
       <c r="K27">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
@@ -2977,35 +3290,35 @@
       </c>
       <c r="B28">
         <f t="shared" si="10"/>
-        <v>18000</v>
+        <v>17250</v>
       </c>
       <c r="C28">
         <f t="shared" si="11"/>
-        <v>24000</v>
+        <v>23000</v>
       </c>
       <c r="D28">
         <f t="shared" si="12"/>
-        <v>2040</v>
+        <v>4275</v>
       </c>
       <c r="E28">
         <f t="shared" si="13"/>
-        <v>61982.649821833504</v>
+        <v>55575</v>
       </c>
       <c r="F28">
         <f t="shared" si="14"/>
-        <v>6120</v>
+        <v>12825</v>
       </c>
       <c r="G28">
         <f t="shared" si="15"/>
-        <v>48120</v>
+        <v>53075</v>
       </c>
       <c r="H28">
         <f t="shared" si="16"/>
-        <v>13862.649821833504</v>
+        <v>2500</v>
       </c>
       <c r="I28">
         <f t="shared" si="9"/>
-        <v>451825.07288629736</v>
+        <v>135000</v>
       </c>
       <c r="J28" t="str">
         <f t="shared" si="7"/>
@@ -3013,7 +3326,7 @@
       </c>
       <c r="K28">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
@@ -3022,35 +3335,35 @@
       </c>
       <c r="B29">
         <f t="shared" si="10"/>
-        <v>18000</v>
+        <v>17250</v>
       </c>
       <c r="C29">
         <f t="shared" si="11"/>
-        <v>24000</v>
+        <v>23000</v>
       </c>
       <c r="D29">
         <f t="shared" si="12"/>
-        <v>2040</v>
+        <v>4275</v>
       </c>
       <c r="E29">
         <f t="shared" si="13"/>
-        <v>61982.649821833504</v>
+        <v>55575</v>
       </c>
       <c r="F29">
         <f t="shared" si="14"/>
-        <v>6120</v>
+        <v>12825</v>
       </c>
       <c r="G29">
         <f t="shared" si="15"/>
-        <v>48120</v>
+        <v>53075</v>
       </c>
       <c r="H29">
         <f t="shared" si="16"/>
-        <v>13862.649821833504</v>
+        <v>2500</v>
       </c>
       <c r="I29">
         <f t="shared" si="9"/>
-        <v>465687.72270813084</v>
+        <v>137500</v>
       </c>
       <c r="J29" t="str">
         <f t="shared" si="7"/>
@@ -3058,7 +3371,7 @@
       </c>
       <c r="K29">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
@@ -3067,35 +3380,35 @@
       </c>
       <c r="B30">
         <f t="shared" si="10"/>
-        <v>18000</v>
+        <v>17250</v>
       </c>
       <c r="C30">
         <f t="shared" si="11"/>
-        <v>24000</v>
+        <v>23000</v>
       </c>
       <c r="D30">
         <f t="shared" si="12"/>
-        <v>2040</v>
+        <v>4275</v>
       </c>
       <c r="E30">
         <f t="shared" si="13"/>
-        <v>61982.649821833504</v>
+        <v>55575</v>
       </c>
       <c r="F30">
         <f t="shared" si="14"/>
-        <v>6120</v>
+        <v>12825</v>
       </c>
       <c r="G30">
         <f t="shared" si="15"/>
-        <v>48120</v>
+        <v>53075</v>
       </c>
       <c r="H30">
         <f t="shared" si="16"/>
-        <v>13862.649821833504</v>
+        <v>2500</v>
       </c>
       <c r="I30">
         <f t="shared" si="9"/>
-        <v>479550.37252996431</v>
+        <v>140000</v>
       </c>
       <c r="J30" t="str">
         <f t="shared" si="7"/>
@@ -3103,7 +3416,7 @@
       </c>
       <c r="K30">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
@@ -3112,35 +3425,35 @@
       </c>
       <c r="B31">
         <f t="shared" si="10"/>
-        <v>18000</v>
+        <v>17250</v>
       </c>
       <c r="C31">
         <f t="shared" si="11"/>
-        <v>24000</v>
+        <v>23000</v>
       </c>
       <c r="D31">
         <f t="shared" si="12"/>
-        <v>2040</v>
+        <v>4275</v>
       </c>
       <c r="E31">
         <f t="shared" si="13"/>
-        <v>61982.649821833504</v>
+        <v>55575</v>
       </c>
       <c r="F31">
         <f t="shared" si="14"/>
-        <v>6120</v>
+        <v>12825</v>
       </c>
       <c r="G31">
         <f t="shared" si="15"/>
-        <v>48120</v>
+        <v>53075</v>
       </c>
       <c r="H31">
         <f t="shared" si="16"/>
-        <v>13862.649821833504</v>
+        <v>2500</v>
       </c>
       <c r="I31">
         <f t="shared" si="9"/>
-        <v>493413.02235179779</v>
+        <v>142500</v>
       </c>
       <c r="J31" t="str">
         <f t="shared" si="7"/>
@@ -3148,7 +3461,7 @@
       </c>
       <c r="K31">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
@@ -3157,35 +3470,35 @@
       </c>
       <c r="B32">
         <f t="shared" si="10"/>
-        <v>18000</v>
+        <v>17250</v>
       </c>
       <c r="C32">
         <f t="shared" si="11"/>
-        <v>24000</v>
+        <v>23000</v>
       </c>
       <c r="D32">
         <f t="shared" si="12"/>
-        <v>2040</v>
+        <v>4275</v>
       </c>
       <c r="E32">
         <f t="shared" si="13"/>
-        <v>61982.649821833504</v>
+        <v>55575</v>
       </c>
       <c r="F32">
         <f t="shared" si="14"/>
-        <v>6120</v>
+        <v>12825</v>
       </c>
       <c r="G32">
         <f t="shared" si="15"/>
-        <v>48120</v>
+        <v>53075</v>
       </c>
       <c r="H32">
         <f t="shared" si="16"/>
-        <v>13862.649821833504</v>
+        <v>2500</v>
       </c>
       <c r="I32">
         <f t="shared" si="9"/>
-        <v>507275.67217363126</v>
+        <v>145000</v>
       </c>
       <c r="J32" t="str">
         <f t="shared" si="7"/>
@@ -3193,7 +3506,7 @@
       </c>
       <c r="K32">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
@@ -3202,35 +3515,35 @@
       </c>
       <c r="B33">
         <f t="shared" si="10"/>
-        <v>18000</v>
+        <v>17250</v>
       </c>
       <c r="C33">
         <f t="shared" si="11"/>
-        <v>24000</v>
+        <v>23000</v>
       </c>
       <c r="D33">
         <f t="shared" si="12"/>
-        <v>2040</v>
+        <v>4275</v>
       </c>
       <c r="E33">
         <f t="shared" si="13"/>
-        <v>61982.649821833504</v>
+        <v>55575</v>
       </c>
       <c r="F33">
         <f t="shared" si="14"/>
-        <v>6120</v>
+        <v>12825</v>
       </c>
       <c r="G33">
         <f t="shared" si="15"/>
-        <v>48120</v>
+        <v>53075</v>
       </c>
       <c r="H33">
         <f t="shared" si="16"/>
-        <v>13862.649821833504</v>
+        <v>2500</v>
       </c>
       <c r="I33">
         <f t="shared" si="9"/>
-        <v>521138.32199546474</v>
+        <v>147500</v>
       </c>
       <c r="J33" t="str">
         <f t="shared" si="7"/>
@@ -3238,7 +3551,7 @@
       </c>
       <c r="K33">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
@@ -3247,35 +3560,35 @@
       </c>
       <c r="B34">
         <f t="shared" si="10"/>
-        <v>18000</v>
+        <v>17250</v>
       </c>
       <c r="C34">
         <f t="shared" si="11"/>
-        <v>24000</v>
+        <v>23000</v>
       </c>
       <c r="D34">
         <f t="shared" si="12"/>
-        <v>2040</v>
+        <v>4275</v>
       </c>
       <c r="E34">
         <f t="shared" si="13"/>
-        <v>61982.649821833504</v>
+        <v>55575</v>
       </c>
       <c r="F34">
         <f t="shared" si="14"/>
-        <v>6120</v>
+        <v>12825</v>
       </c>
       <c r="G34">
         <f t="shared" si="15"/>
-        <v>48120</v>
+        <v>53075</v>
       </c>
       <c r="H34">
         <f t="shared" si="16"/>
-        <v>13862.649821833504</v>
+        <v>2500</v>
       </c>
       <c r="I34">
         <f t="shared" si="9"/>
-        <v>535000.97181729821</v>
+        <v>150000</v>
       </c>
       <c r="J34" t="str">
         <f t="shared" si="7"/>
@@ -3283,7 +3596,7 @@
       </c>
       <c r="K34">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
@@ -3292,35 +3605,35 @@
       </c>
       <c r="B35">
         <f>$B$23*(1+$B$7)</f>
-        <v>21600</v>
+        <v>19837.5</v>
       </c>
       <c r="C35">
         <f>C23*(1+$B$7)</f>
-        <v>28800</v>
+        <v>26449.999999999996</v>
       </c>
       <c r="D35">
         <f>D23*(1+$B$8)</f>
-        <v>1734</v>
+        <v>4061.25</v>
       </c>
       <c r="E35">
         <f t="shared" si="13"/>
-        <v>52685.252348558475</v>
+        <v>52796.25</v>
       </c>
       <c r="F35">
         <f t="shared" si="14"/>
-        <v>5202</v>
+        <v>12183.75</v>
       </c>
       <c r="G35">
         <f t="shared" si="15"/>
-        <v>55602</v>
+        <v>58471.25</v>
       </c>
       <c r="H35">
         <f t="shared" si="16"/>
-        <v>-2916.7476514415248</v>
+        <v>-5675</v>
       </c>
       <c r="I35">
         <f t="shared" si="9"/>
-        <v>532084.22416585672</v>
+        <v>144325</v>
       </c>
       <c r="J35" s="2" t="str">
         <f t="shared" si="7"/>
@@ -3337,35 +3650,35 @@
       </c>
       <c r="B36">
         <f t="shared" ref="B36:B46" si="17">$B$23*(1+$B$7)</f>
-        <v>21600</v>
+        <v>19837.5</v>
       </c>
       <c r="C36">
         <f t="shared" ref="C36:C46" si="18">C24*(1+$B$7)</f>
-        <v>28800</v>
+        <v>26449.999999999996</v>
       </c>
       <c r="D36">
         <f t="shared" ref="D36:D46" si="19">D24*(1+$B$8)</f>
-        <v>1734</v>
+        <v>4061.25</v>
       </c>
       <c r="E36">
         <f t="shared" si="13"/>
-        <v>52685.252348558475</v>
+        <v>52796.25</v>
       </c>
       <c r="F36">
         <f t="shared" si="14"/>
-        <v>5202</v>
+        <v>12183.75</v>
       </c>
       <c r="G36">
         <f t="shared" si="15"/>
-        <v>55602</v>
+        <v>58471.25</v>
       </c>
       <c r="H36">
         <f t="shared" si="16"/>
-        <v>-2916.7476514415248</v>
+        <v>-5675</v>
       </c>
       <c r="I36">
         <f t="shared" si="9"/>
-        <v>529167.47651441523</v>
+        <v>138650</v>
       </c>
       <c r="J36" s="2" t="str">
         <f t="shared" si="7"/>
@@ -3382,35 +3695,35 @@
       </c>
       <c r="B37">
         <f t="shared" si="17"/>
-        <v>21600</v>
+        <v>19837.5</v>
       </c>
       <c r="C37">
         <f t="shared" si="18"/>
-        <v>28800</v>
+        <v>26449.999999999996</v>
       </c>
       <c r="D37">
         <f t="shared" si="19"/>
-        <v>1734</v>
+        <v>4061.25</v>
       </c>
       <c r="E37">
         <f t="shared" si="13"/>
-        <v>52685.252348558475</v>
+        <v>52796.25</v>
       </c>
       <c r="F37">
         <f t="shared" si="14"/>
-        <v>5202</v>
+        <v>12183.75</v>
       </c>
       <c r="G37">
         <f t="shared" si="15"/>
-        <v>55602</v>
+        <v>58471.25</v>
       </c>
       <c r="H37">
         <f t="shared" si="16"/>
-        <v>-2916.7476514415248</v>
+        <v>-5675</v>
       </c>
       <c r="I37">
         <f t="shared" si="9"/>
-        <v>526250.72886297374</v>
+        <v>132975</v>
       </c>
       <c r="J37" s="2" t="str">
         <f t="shared" si="7"/>
@@ -3427,35 +3740,35 @@
       </c>
       <c r="B38">
         <f t="shared" si="17"/>
-        <v>21600</v>
+        <v>19837.5</v>
       </c>
       <c r="C38">
         <f t="shared" si="18"/>
-        <v>28800</v>
+        <v>26449.999999999996</v>
       </c>
       <c r="D38">
         <f t="shared" si="19"/>
-        <v>1734</v>
+        <v>4061.25</v>
       </c>
       <c r="E38">
         <f t="shared" si="13"/>
-        <v>52685.252348558475</v>
+        <v>52796.25</v>
       </c>
       <c r="F38">
         <f t="shared" si="14"/>
-        <v>5202</v>
+        <v>12183.75</v>
       </c>
       <c r="G38">
         <f t="shared" si="15"/>
-        <v>55602</v>
+        <v>58471.25</v>
       </c>
       <c r="H38">
         <f t="shared" si="16"/>
-        <v>-2916.7476514415248</v>
+        <v>-5675</v>
       </c>
       <c r="I38">
         <f t="shared" si="9"/>
-        <v>523333.9812115322</v>
+        <v>127300</v>
       </c>
       <c r="J38" s="2" t="str">
         <f t="shared" si="7"/>
@@ -3472,35 +3785,35 @@
       </c>
       <c r="B39">
         <f t="shared" si="17"/>
-        <v>21600</v>
+        <v>19837.5</v>
       </c>
       <c r="C39">
         <f t="shared" si="18"/>
-        <v>28800</v>
+        <v>26449.999999999996</v>
       </c>
       <c r="D39">
         <f t="shared" si="19"/>
-        <v>1734</v>
+        <v>4061.25</v>
       </c>
       <c r="E39">
         <f t="shared" si="13"/>
-        <v>52685.252348558475</v>
+        <v>52796.25</v>
       </c>
       <c r="F39">
         <f t="shared" si="14"/>
-        <v>5202</v>
+        <v>12183.75</v>
       </c>
       <c r="G39">
         <f t="shared" si="15"/>
-        <v>55602</v>
+        <v>58471.25</v>
       </c>
       <c r="H39">
         <f t="shared" si="16"/>
-        <v>-2916.7476514415248</v>
+        <v>-5675</v>
       </c>
       <c r="I39">
         <f t="shared" si="9"/>
-        <v>520417.23356009065</v>
+        <v>121625</v>
       </c>
       <c r="J39" s="2" t="str">
         <f t="shared" si="7"/>
@@ -3517,35 +3830,35 @@
       </c>
       <c r="B40">
         <f t="shared" si="17"/>
-        <v>21600</v>
+        <v>19837.5</v>
       </c>
       <c r="C40">
         <f t="shared" si="18"/>
-        <v>28800</v>
+        <v>26449.999999999996</v>
       </c>
       <c r="D40">
         <f t="shared" si="19"/>
-        <v>1734</v>
+        <v>4061.25</v>
       </c>
       <c r="E40">
         <f t="shared" si="13"/>
-        <v>52685.252348558475</v>
+        <v>52796.25</v>
       </c>
       <c r="F40">
         <f t="shared" si="14"/>
-        <v>5202</v>
+        <v>12183.75</v>
       </c>
       <c r="G40">
         <f t="shared" si="15"/>
-        <v>55602</v>
+        <v>58471.25</v>
       </c>
       <c r="H40">
         <f t="shared" si="16"/>
-        <v>-2916.7476514415248</v>
+        <v>-5675</v>
       </c>
       <c r="I40">
         <f t="shared" si="9"/>
-        <v>517500.48590864911</v>
+        <v>115950</v>
       </c>
       <c r="J40" s="2" t="str">
         <f t="shared" si="7"/>
@@ -3562,35 +3875,35 @@
       </c>
       <c r="B41">
         <f t="shared" si="17"/>
-        <v>21600</v>
+        <v>19837.5</v>
       </c>
       <c r="C41">
         <f t="shared" si="18"/>
-        <v>28800</v>
+        <v>26449.999999999996</v>
       </c>
       <c r="D41">
         <f t="shared" si="19"/>
-        <v>1734</v>
+        <v>4061.25</v>
       </c>
       <c r="E41">
         <f t="shared" si="13"/>
-        <v>52685.252348558475</v>
+        <v>52796.25</v>
       </c>
       <c r="F41">
         <f t="shared" si="14"/>
-        <v>5202</v>
+        <v>12183.75</v>
       </c>
       <c r="G41">
         <f t="shared" si="15"/>
-        <v>55602</v>
+        <v>58471.25</v>
       </c>
       <c r="H41">
         <f t="shared" si="16"/>
-        <v>-2916.7476514415248</v>
+        <v>-5675</v>
       </c>
       <c r="I41">
         <f t="shared" si="9"/>
-        <v>514583.73825720756</v>
+        <v>110275</v>
       </c>
       <c r="J41" s="2" t="str">
         <f t="shared" si="7"/>
@@ -3607,35 +3920,35 @@
       </c>
       <c r="B42">
         <f t="shared" si="17"/>
-        <v>21600</v>
+        <v>19837.5</v>
       </c>
       <c r="C42">
         <f t="shared" si="18"/>
-        <v>28800</v>
+        <v>26449.999999999996</v>
       </c>
       <c r="D42">
         <f t="shared" si="19"/>
-        <v>1734</v>
+        <v>4061.25</v>
       </c>
       <c r="E42">
         <f t="shared" si="13"/>
-        <v>52685.252348558475</v>
+        <v>52796.25</v>
       </c>
       <c r="F42">
         <f t="shared" si="14"/>
-        <v>5202</v>
+        <v>12183.75</v>
       </c>
       <c r="G42">
         <f t="shared" si="15"/>
-        <v>55602</v>
+        <v>58471.25</v>
       </c>
       <c r="H42">
         <f t="shared" si="16"/>
-        <v>-2916.7476514415248</v>
+        <v>-5675</v>
       </c>
       <c r="I42">
         <f t="shared" si="9"/>
-        <v>511666.99060576601</v>
+        <v>104600</v>
       </c>
       <c r="J42" s="2" t="str">
         <f t="shared" si="7"/>
@@ -3652,35 +3965,35 @@
       </c>
       <c r="B43">
         <f t="shared" si="17"/>
-        <v>21600</v>
+        <v>19837.5</v>
       </c>
       <c r="C43">
         <f t="shared" si="18"/>
-        <v>28800</v>
+        <v>26449.999999999996</v>
       </c>
       <c r="D43">
         <f t="shared" si="19"/>
-        <v>1734</v>
+        <v>4061.25</v>
       </c>
       <c r="E43">
         <f t="shared" si="13"/>
-        <v>52685.252348558475</v>
+        <v>52796.25</v>
       </c>
       <c r="F43">
         <f t="shared" si="14"/>
-        <v>5202</v>
+        <v>12183.75</v>
       </c>
       <c r="G43">
         <f t="shared" si="15"/>
-        <v>55602</v>
+        <v>58471.25</v>
       </c>
       <c r="H43">
         <f t="shared" si="16"/>
-        <v>-2916.7476514415248</v>
+        <v>-5675</v>
       </c>
       <c r="I43">
         <f t="shared" si="9"/>
-        <v>508750.24295432447</v>
+        <v>98925</v>
       </c>
       <c r="J43" s="2" t="str">
         <f t="shared" si="7"/>
@@ -3697,35 +4010,35 @@
       </c>
       <c r="B44">
         <f t="shared" si="17"/>
-        <v>21600</v>
+        <v>19837.5</v>
       </c>
       <c r="C44">
         <f t="shared" si="18"/>
-        <v>28800</v>
+        <v>26449.999999999996</v>
       </c>
       <c r="D44">
         <f t="shared" si="19"/>
-        <v>1734</v>
+        <v>4061.25</v>
       </c>
       <c r="E44">
         <f t="shared" si="13"/>
-        <v>52685.252348558475</v>
+        <v>52796.25</v>
       </c>
       <c r="F44">
         <f t="shared" si="14"/>
-        <v>5202</v>
+        <v>12183.75</v>
       </c>
       <c r="G44">
         <f t="shared" si="15"/>
-        <v>55602</v>
+        <v>58471.25</v>
       </c>
       <c r="H44">
         <f t="shared" si="16"/>
-        <v>-2916.7476514415248</v>
+        <v>-5675</v>
       </c>
       <c r="I44">
         <f t="shared" si="9"/>
-        <v>505833.49530288292</v>
+        <v>93250</v>
       </c>
       <c r="J44" s="2" t="str">
         <f t="shared" si="7"/>
@@ -3742,35 +4055,35 @@
       </c>
       <c r="B45">
         <f t="shared" si="17"/>
-        <v>21600</v>
+        <v>19837.5</v>
       </c>
       <c r="C45">
         <f t="shared" si="18"/>
-        <v>28800</v>
+        <v>26449.999999999996</v>
       </c>
       <c r="D45">
         <f t="shared" si="19"/>
-        <v>1734</v>
+        <v>4061.25</v>
       </c>
       <c r="E45">
         <f t="shared" si="13"/>
-        <v>52685.252348558475</v>
+        <v>52796.25</v>
       </c>
       <c r="F45">
         <f t="shared" si="14"/>
-        <v>5202</v>
+        <v>12183.75</v>
       </c>
       <c r="G45">
         <f t="shared" si="15"/>
-        <v>55602</v>
+        <v>58471.25</v>
       </c>
       <c r="H45">
         <f t="shared" si="16"/>
-        <v>-2916.7476514415248</v>
+        <v>-5675</v>
       </c>
       <c r="I45">
         <f t="shared" si="9"/>
-        <v>502916.74765144137</v>
+        <v>87575</v>
       </c>
       <c r="J45" s="2" t="str">
         <f t="shared" si="7"/>
@@ -3787,35 +4100,35 @@
       </c>
       <c r="B46">
         <f t="shared" si="17"/>
-        <v>21600</v>
+        <v>19837.5</v>
       </c>
       <c r="C46">
         <f t="shared" si="18"/>
-        <v>28800</v>
+        <v>26449.999999999996</v>
       </c>
       <c r="D46">
         <f t="shared" si="19"/>
-        <v>1734</v>
+        <v>4061.25</v>
       </c>
       <c r="E46">
         <f t="shared" si="13"/>
-        <v>52685.252348558475</v>
+        <v>52796.25</v>
       </c>
       <c r="F46">
         <f t="shared" si="14"/>
-        <v>5202</v>
+        <v>12183.75</v>
       </c>
       <c r="G46">
         <f t="shared" si="15"/>
-        <v>55602</v>
+        <v>58471.25</v>
       </c>
       <c r="H46">
         <f t="shared" si="16"/>
-        <v>-2916.7476514415248</v>
+        <v>-5675</v>
       </c>
       <c r="I46">
         <f t="shared" si="9"/>
-        <v>499999.99999999983</v>
+        <v>81900</v>
       </c>
       <c r="J46" s="2" t="str">
         <f t="shared" si="7"/>

</xml_diff>